<commit_message>
Update Definition of mental health literacy in bcio_moa.xlsx
</commit_message>
<xml_diff>
--- a/MechanismOfAction/bcio_moa.xlsx
+++ b/MechanismOfAction/bcio_moa.xlsx
@@ -24189,7 +24189,7 @@
       </c>
       <c r="C399" s="4" t="inlineStr">
         <is>
-          <t>A &lt;health literacy&gt; concerning mental health.</t>
+          <t>&lt;Health literacy&gt; concerning mental health.</t>
         </is>
       </c>
       <c r="D399" s="4" t="inlineStr">
@@ -24197,32 +24197,32 @@
           <t>health literacy</t>
         </is>
       </c>
-      <c r="E399" s="4" t="inlineStr"/>
-      <c r="F399" s="4" t="inlineStr"/>
-      <c r="G399" s="4" t="inlineStr"/>
-      <c r="H399" s="4" t="inlineStr"/>
-      <c r="I399" s="4" t="inlineStr"/>
-      <c r="J399" s="4" t="inlineStr"/>
-      <c r="K399" s="4" t="inlineStr"/>
-      <c r="L399" s="4" t="inlineStr"/>
-      <c r="M399" s="4" t="inlineStr"/>
-      <c r="N399" s="4" t="inlineStr"/>
-      <c r="O399" s="4" t="inlineStr"/>
-      <c r="P399" s="4" t="inlineStr"/>
-      <c r="Q399" s="4" t="inlineStr"/>
-      <c r="R399" s="4" t="inlineStr"/>
+      <c r="E399" s="4" t="n"/>
+      <c r="F399" s="4" t="n"/>
+      <c r="G399" s="4" t="n"/>
+      <c r="H399" s="4" t="n"/>
+      <c r="I399" s="4" t="n"/>
+      <c r="J399" s="4" t="n"/>
+      <c r="K399" s="4" t="n"/>
+      <c r="L399" s="4" t="n"/>
+      <c r="M399" s="4" t="n"/>
+      <c r="N399" s="4" t="n"/>
+      <c r="O399" s="4" t="n"/>
+      <c r="P399" s="4" t="n"/>
+      <c r="Q399" s="4" t="n"/>
+      <c r="R399" s="4" t="n"/>
       <c r="S399" s="4" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T399" s="4" t="inlineStr"/>
-      <c r="U399" s="4" t="inlineStr"/>
-      <c r="V399" s="4" t="inlineStr"/>
+      <c r="T399" s="4" t="n"/>
+      <c r="U399" s="4" t="n"/>
+      <c r="V399" s="4" t="n"/>
       <c r="W399" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X399" s="4" t="inlineStr"/>
+      <c r="X399" s="4" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Edit bcio_moa.xlsx: update 8, add 2
</commit_message>
<xml_diff>
--- a/MechanismOfAction/bcio_moa.xlsx
+++ b/MechanismOfAction/bcio_moa.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X652"/>
+  <dimension ref="A1:X654"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -562,36 +562,36 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr"/>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Proposed</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr"/>
-      <c r="U2" s="2" t="inlineStr"/>
-      <c r="V2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
       <c r="W2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="X2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -27053,52 +27053,52 @@
       <c r="X448" s="4" t="n"/>
     </row>
     <row r="449">
-      <c r="A449" s="2" t="inlineStr">
+      <c r="A449" s="4" t="inlineStr">
         <is>
           <t>BCIO:051035</t>
         </is>
       </c>
-      <c r="B449" s="2" t="inlineStr">
+      <c r="B449" s="4" t="inlineStr">
         <is>
           <t>negative punishment process</t>
         </is>
       </c>
-      <c r="C449" s="2" t="inlineStr">
+      <c r="C449" s="4" t="inlineStr">
         <is>
           <t>A &lt;punishment process&gt; in which the likelihood of a behaviour is decreased by it being followed by termination or avoidance of a stimulus.</t>
         </is>
       </c>
-      <c r="D449" s="2" t="inlineStr">
+      <c r="D449" s="4" t="inlineStr">
         <is>
           <t>punishment process</t>
         </is>
       </c>
-      <c r="E449" s="2" t="n"/>
-      <c r="F449" s="2" t="n"/>
-      <c r="G449" s="2" t="n"/>
-      <c r="H449" s="2" t="n"/>
-      <c r="I449" s="2" t="n"/>
-      <c r="J449" s="2" t="n"/>
-      <c r="K449" s="2" t="n"/>
-      <c r="L449" s="2" t="n"/>
-      <c r="M449" s="2" t="n"/>
-      <c r="N449" s="2" t="n"/>
-      <c r="O449" s="2" t="n"/>
-      <c r="P449" s="2" t="n"/>
-      <c r="Q449" s="2" t="n"/>
-      <c r="R449" s="2" t="n"/>
-      <c r="S449" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T449" s="2" t="n"/>
-      <c r="U449" s="2" t="n"/>
-      <c r="V449" s="2" t="n"/>
-      <c r="W449" s="2" t="n">
+      <c r="E449" s="4" t="n"/>
+      <c r="F449" s="4" t="n"/>
+      <c r="G449" s="4" t="n"/>
+      <c r="H449" s="4" t="n"/>
+      <c r="I449" s="4" t="n"/>
+      <c r="J449" s="4" t="n"/>
+      <c r="K449" s="4" t="n"/>
+      <c r="L449" s="4" t="n"/>
+      <c r="M449" s="4" t="n"/>
+      <c r="N449" s="4" t="n"/>
+      <c r="O449" s="4" t="n"/>
+      <c r="P449" s="4" t="n"/>
+      <c r="Q449" s="4" t="n"/>
+      <c r="R449" s="4" t="n"/>
+      <c r="S449" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T449" s="4" t="n"/>
+      <c r="U449" s="4" t="n"/>
+      <c r="V449" s="4" t="n"/>
+      <c r="W449" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X449" s="2" t="n"/>
+      <c r="X449" s="4" t="n"/>
     </row>
     <row r="450">
       <c r="A450" s="4" t="inlineStr">
@@ -30182,52 +30182,52 @@
       <c r="X500" s="4" t="n"/>
     </row>
     <row r="501">
-      <c r="A501" s="2" t="inlineStr">
+      <c r="A501" s="4" t="inlineStr">
         <is>
           <t>BCIO:051037</t>
         </is>
       </c>
-      <c r="B501" s="2" t="inlineStr">
+      <c r="B501" s="4" t="inlineStr">
         <is>
           <t>positive punishment process</t>
         </is>
       </c>
-      <c r="C501" s="2" t="inlineStr">
+      <c r="C501" s="4" t="inlineStr">
         <is>
           <t>A &lt;punishment process&gt; in which the likelihood of a behaviour is decreased by it being followed by a stimulus.</t>
         </is>
       </c>
-      <c r="D501" s="2" t="inlineStr">
+      <c r="D501" s="4" t="inlineStr">
         <is>
           <t>punishment process</t>
         </is>
       </c>
-      <c r="E501" s="2" t="n"/>
-      <c r="F501" s="2" t="n"/>
-      <c r="G501" s="2" t="n"/>
-      <c r="H501" s="2" t="n"/>
-      <c r="I501" s="2" t="n"/>
-      <c r="J501" s="2" t="n"/>
-      <c r="K501" s="2" t="n"/>
-      <c r="L501" s="2" t="n"/>
-      <c r="M501" s="2" t="n"/>
-      <c r="N501" s="2" t="n"/>
-      <c r="O501" s="2" t="n"/>
-      <c r="P501" s="2" t="n"/>
-      <c r="Q501" s="2" t="n"/>
-      <c r="R501" s="2" t="n"/>
-      <c r="S501" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T501" s="2" t="n"/>
-      <c r="U501" s="2" t="n"/>
-      <c r="V501" s="2" t="n"/>
-      <c r="W501" s="2" t="n">
+      <c r="E501" s="4" t="n"/>
+      <c r="F501" s="4" t="n"/>
+      <c r="G501" s="4" t="n"/>
+      <c r="H501" s="4" t="n"/>
+      <c r="I501" s="4" t="n"/>
+      <c r="J501" s="4" t="n"/>
+      <c r="K501" s="4" t="n"/>
+      <c r="L501" s="4" t="n"/>
+      <c r="M501" s="4" t="n"/>
+      <c r="N501" s="4" t="n"/>
+      <c r="O501" s="4" t="n"/>
+      <c r="P501" s="4" t="n"/>
+      <c r="Q501" s="4" t="n"/>
+      <c r="R501" s="4" t="n"/>
+      <c r="S501" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T501" s="4" t="n"/>
+      <c r="U501" s="4" t="n"/>
+      <c r="V501" s="4" t="n"/>
+      <c r="W501" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X501" s="2" t="n"/>
+      <c r="X501" s="4" t="n"/>
     </row>
     <row r="502">
       <c r="A502" s="4" t="inlineStr">
@@ -30559,163 +30559,163 @@
       <c r="X507" s="4" t="n"/>
     </row>
     <row r="508">
-      <c r="A508" s="2" t="inlineStr">
+      <c r="A508" s="4" t="inlineStr">
         <is>
           <t>BCIO:051039</t>
         </is>
       </c>
-      <c r="B508" s="2" t="inlineStr">
+      <c r="B508" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">primary punishing stimulus
 </t>
         </is>
       </c>
-      <c r="C508" s="2" t="inlineStr">
+      <c r="C508" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">A &lt;punishing stimulus&gt; whose effect on behaviour derives from the animal’s genotype rather than being learned by association with another stimulus. </t>
         </is>
       </c>
-      <c r="D508" s="2" t="inlineStr">
+      <c r="D508" s="4" t="inlineStr">
         <is>
           <t>punishing stimulus</t>
         </is>
       </c>
-      <c r="E508" s="2" t="inlineStr"/>
-      <c r="F508" s="2" t="inlineStr"/>
-      <c r="G508" s="2" t="inlineStr"/>
-      <c r="H508" s="2" t="inlineStr"/>
-      <c r="I508" s="2" t="inlineStr"/>
-      <c r="J508" s="2" t="inlineStr"/>
-      <c r="K508" s="2" t="inlineStr"/>
-      <c r="L508" s="2" t="inlineStr"/>
-      <c r="M508" s="2" t="inlineStr"/>
-      <c r="N508" s="2" t="inlineStr"/>
-      <c r="O508" s="2" t="inlineStr"/>
-      <c r="P508" s="2" t="inlineStr"/>
-      <c r="Q508" s="2" t="inlineStr"/>
-      <c r="R508" s="2" t="inlineStr"/>
-      <c r="S508" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T508" s="2" t="inlineStr"/>
-      <c r="U508" s="2" t="inlineStr"/>
-      <c r="V508" s="2" t="inlineStr"/>
-      <c r="W508" s="2" t="n">
+      <c r="E508" s="4" t="n"/>
+      <c r="F508" s="4" t="n"/>
+      <c r="G508" s="4" t="n"/>
+      <c r="H508" s="4" t="n"/>
+      <c r="I508" s="4" t="n"/>
+      <c r="J508" s="4" t="n"/>
+      <c r="K508" s="4" t="n"/>
+      <c r="L508" s="4" t="n"/>
+      <c r="M508" s="4" t="n"/>
+      <c r="N508" s="4" t="n"/>
+      <c r="O508" s="4" t="n"/>
+      <c r="P508" s="4" t="n"/>
+      <c r="Q508" s="4" t="n"/>
+      <c r="R508" s="4" t="n"/>
+      <c r="S508" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T508" s="4" t="n"/>
+      <c r="U508" s="4" t="n"/>
+      <c r="V508" s="4" t="n"/>
+      <c r="W508" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X508" s="2" t="inlineStr"/>
+      <c r="X508" s="4" t="n"/>
     </row>
     <row r="509">
-      <c r="A509" s="4" t="inlineStr">
+      <c r="A509" s="3" t="inlineStr">
         <is>
           <t>BCIO:050741</t>
         </is>
       </c>
-      <c r="B509" s="4" t="inlineStr">
+      <c r="B509" s="3" t="inlineStr">
         <is>
           <t>primary reinforcer</t>
         </is>
       </c>
-      <c r="C509" s="4" t="inlineStr">
+      <c r="C509" s="3" t="inlineStr">
         <is>
           <t>A &lt;reinforcer&gt; whose effect on behaviour is innately determined.</t>
         </is>
       </c>
-      <c r="D509" s="4" t="inlineStr">
+      <c r="D509" s="3" t="inlineStr">
         <is>
           <t>reinforcer</t>
         </is>
       </c>
-      <c r="E509" s="4" t="n"/>
-      <c r="F509" s="4" t="n"/>
-      <c r="G509" s="4" t="inlineStr">
+      <c r="E509" s="3" t="n"/>
+      <c r="F509" s="3" t="n"/>
+      <c r="G509" s="3" t="inlineStr">
         <is>
           <t>"Positive reinforcement" in the Operant Conditioning; "Innate rewards" in the Social Learning Theory</t>
         </is>
       </c>
-      <c r="H509" s="4" t="n"/>
-      <c r="I509" s="4" t="n"/>
-      <c r="J509" s="4" t="n"/>
-      <c r="K509" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L509" s="4" t="n"/>
-      <c r="M509" s="4" t="n"/>
-      <c r="N509" s="4" t="n"/>
-      <c r="O509" s="4" t="n"/>
-      <c r="P509" s="4" t="n"/>
-      <c r="Q509" s="4" t="n"/>
-      <c r="R509" s="4" t="n"/>
-      <c r="S509" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T509" s="4" t="n"/>
-      <c r="U509" s="4" t="n"/>
-      <c r="V509" s="4" t="inlineStr">
+      <c r="H509" s="3" t="n"/>
+      <c r="I509" s="3" t="n"/>
+      <c r="J509" s="3" t="n"/>
+      <c r="K509" s="3" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L509" s="3" t="n"/>
+      <c r="M509" s="3" t="n"/>
+      <c r="N509" s="3" t="n"/>
+      <c r="O509" s="3" t="n"/>
+      <c r="P509" s="3" t="n"/>
+      <c r="Q509" s="3" t="n"/>
+      <c r="R509" s="3" t="n"/>
+      <c r="S509" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="T509" s="3" t="n"/>
+      <c r="U509" s="3" t="n"/>
+      <c r="V509" s="3" t="inlineStr">
         <is>
           <t>PS; LZ; JD</t>
         </is>
       </c>
-      <c r="W509" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X509" s="4" t="n"/>
+      <c r="W509" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X509" s="3" t="n"/>
     </row>
     <row r="510">
-      <c r="A510" s="2" t="inlineStr">
+      <c r="A510" s="4" t="inlineStr">
         <is>
           <t>BCIO:051040</t>
         </is>
       </c>
-      <c r="B510" s="2" t="inlineStr">
+      <c r="B510" s="4" t="inlineStr">
         <is>
           <t>primary reinforcer</t>
         </is>
       </c>
-      <c r="C510" s="2" t="inlineStr">
+      <c r="C510" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> A &lt;reinforcer&gt; whose effect on behaviour derives from the animal’s genotype rather than being learned by association with another stimulus.</t>
         </is>
       </c>
-      <c r="D510" s="2" t="inlineStr">
+      <c r="D510" s="4" t="inlineStr">
         <is>
           <t>reinforcer</t>
         </is>
       </c>
-      <c r="E510" s="2" t="inlineStr"/>
-      <c r="F510" s="2" t="inlineStr"/>
-      <c r="G510" s="2" t="inlineStr"/>
-      <c r="H510" s="2" t="inlineStr"/>
-      <c r="I510" s="2" t="inlineStr"/>
-      <c r="J510" s="2" t="inlineStr"/>
-      <c r="K510" s="2" t="inlineStr"/>
-      <c r="L510" s="2" t="inlineStr"/>
-      <c r="M510" s="2" t="inlineStr"/>
-      <c r="N510" s="2" t="inlineStr"/>
-      <c r="O510" s="2" t="inlineStr"/>
-      <c r="P510" s="2" t="inlineStr"/>
-      <c r="Q510" s="2" t="inlineStr"/>
-      <c r="R510" s="2" t="inlineStr"/>
-      <c r="S510" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T510" s="2" t="inlineStr"/>
-      <c r="U510" s="2" t="inlineStr"/>
-      <c r="V510" s="2" t="inlineStr"/>
-      <c r="W510" s="2" t="n">
+      <c r="E510" s="4" t="n"/>
+      <c r="F510" s="4" t="n"/>
+      <c r="G510" s="4" t="n"/>
+      <c r="H510" s="4" t="n"/>
+      <c r="I510" s="4" t="n"/>
+      <c r="J510" s="4" t="n"/>
+      <c r="K510" s="4" t="n"/>
+      <c r="L510" s="4" t="n"/>
+      <c r="M510" s="4" t="n"/>
+      <c r="N510" s="4" t="n"/>
+      <c r="O510" s="4" t="n"/>
+      <c r="P510" s="4" t="n"/>
+      <c r="Q510" s="4" t="n"/>
+      <c r="R510" s="4" t="n"/>
+      <c r="S510" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T510" s="4" t="n"/>
+      <c r="U510" s="4" t="n"/>
+      <c r="V510" s="4" t="n"/>
+      <c r="W510" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X510" s="2" t="inlineStr"/>
+      <c r="X510" s="4" t="n"/>
     </row>
     <row r="511">
       <c r="A511" s="4" t="inlineStr">
@@ -31778,52 +31778,52 @@
       <c r="X527" s="4" t="n"/>
     </row>
     <row r="528">
-      <c r="A528" s="2" t="inlineStr">
+      <c r="A528" s="4" t="inlineStr">
         <is>
           <t>BCIO:051033</t>
         </is>
       </c>
-      <c r="B528" s="2" t="inlineStr">
+      <c r="B528" s="4" t="inlineStr">
         <is>
           <t>punishment process</t>
         </is>
       </c>
-      <c r="C528" s="2" t="inlineStr">
+      <c r="C528" s="4" t="inlineStr">
         <is>
           <t>A &lt;behavioural contingency process&gt; in which a behaviour is followed by a stimulus that decreases the likelihood of occurrence of the behaviour.</t>
         </is>
       </c>
-      <c r="D528" s="2" t="inlineStr">
+      <c r="D528" s="4" t="inlineStr">
         <is>
           <t>behavioural contingency process</t>
         </is>
       </c>
-      <c r="E528" s="2" t="n"/>
-      <c r="F528" s="2" t="n"/>
-      <c r="G528" s="2" t="n"/>
-      <c r="H528" s="2" t="n"/>
-      <c r="I528" s="2" t="n"/>
-      <c r="J528" s="2" t="n"/>
-      <c r="K528" s="2" t="n"/>
-      <c r="L528" s="2" t="n"/>
-      <c r="M528" s="2" t="n"/>
-      <c r="N528" s="2" t="n"/>
-      <c r="O528" s="2" t="n"/>
-      <c r="P528" s="2" t="n"/>
-      <c r="Q528" s="2" t="n"/>
-      <c r="R528" s="2" t="n"/>
-      <c r="S528" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T528" s="2" t="n"/>
-      <c r="U528" s="2" t="n"/>
-      <c r="V528" s="2" t="n"/>
-      <c r="W528" s="2" t="n">
+      <c r="E528" s="4" t="n"/>
+      <c r="F528" s="4" t="n"/>
+      <c r="G528" s="4" t="n"/>
+      <c r="H528" s="4" t="n"/>
+      <c r="I528" s="4" t="n"/>
+      <c r="J528" s="4" t="n"/>
+      <c r="K528" s="4" t="n"/>
+      <c r="L528" s="4" t="n"/>
+      <c r="M528" s="4" t="n"/>
+      <c r="N528" s="4" t="n"/>
+      <c r="O528" s="4" t="n"/>
+      <c r="P528" s="4" t="n"/>
+      <c r="Q528" s="4" t="n"/>
+      <c r="R528" s="4" t="n"/>
+      <c r="S528" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T528" s="4" t="n"/>
+      <c r="U528" s="4" t="n"/>
+      <c r="V528" s="4" t="n"/>
+      <c r="W528" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X528" s="2" t="n"/>
+      <c r="X528" s="4" t="n"/>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
@@ -32302,52 +32302,52 @@
       <c r="X536" s="4" t="n"/>
     </row>
     <row r="537">
-      <c r="A537" s="2" t="inlineStr">
+      <c r="A537" s="4" t="inlineStr">
         <is>
           <t>BCIO:051034</t>
         </is>
       </c>
-      <c r="B537" s="2" t="inlineStr">
+      <c r="B537" s="4" t="inlineStr">
         <is>
           <t>reinforcement process</t>
         </is>
       </c>
-      <c r="C537" s="2" t="inlineStr">
+      <c r="C537" s="4" t="inlineStr">
         <is>
           <t>A &lt;behavioural contingency process&gt; in which a behaviour is followed by a stimulus that increases the likelihood of occurrence of the behaviour.</t>
         </is>
       </c>
-      <c r="D537" s="2" t="inlineStr">
+      <c r="D537" s="4" t="inlineStr">
         <is>
           <t>behavioural contingency process</t>
         </is>
       </c>
-      <c r="E537" s="2" t="n"/>
-      <c r="F537" s="2" t="n"/>
-      <c r="G537" s="2" t="n"/>
-      <c r="H537" s="2" t="n"/>
-      <c r="I537" s="2" t="n"/>
-      <c r="J537" s="2" t="n"/>
-      <c r="K537" s="2" t="n"/>
-      <c r="L537" s="2" t="n"/>
-      <c r="M537" s="2" t="n"/>
-      <c r="N537" s="2" t="n"/>
-      <c r="O537" s="2" t="n"/>
-      <c r="P537" s="2" t="n"/>
-      <c r="Q537" s="2" t="n"/>
-      <c r="R537" s="2" t="n"/>
-      <c r="S537" s="2" t="inlineStr">
-        <is>
-          <t>Proposed</t>
-        </is>
-      </c>
-      <c r="T537" s="2" t="n"/>
-      <c r="U537" s="2" t="n"/>
-      <c r="V537" s="2" t="n"/>
-      <c r="W537" s="2" t="n">
+      <c r="E537" s="4" t="n"/>
+      <c r="F537" s="4" t="n"/>
+      <c r="G537" s="4" t="n"/>
+      <c r="H537" s="4" t="n"/>
+      <c r="I537" s="4" t="n"/>
+      <c r="J537" s="4" t="n"/>
+      <c r="K537" s="4" t="n"/>
+      <c r="L537" s="4" t="n"/>
+      <c r="M537" s="4" t="n"/>
+      <c r="N537" s="4" t="n"/>
+      <c r="O537" s="4" t="n"/>
+      <c r="P537" s="4" t="n"/>
+      <c r="Q537" s="4" t="n"/>
+      <c r="R537" s="4" t="n"/>
+      <c r="S537" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T537" s="4" t="n"/>
+      <c r="U537" s="4" t="n"/>
+      <c r="V537" s="4" t="n"/>
+      <c r="W537" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X537" s="2" t="n"/>
+      <c r="X537" s="4" t="n"/>
     </row>
     <row r="538">
       <c r="A538" s="4" t="inlineStr">
@@ -36252,220 +36252,192 @@
     <row r="604">
       <c r="A604" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050778</t>
+          <t>BCIO:051041</t>
         </is>
       </c>
       <c r="B604" s="4" t="inlineStr">
         <is>
-          <t>social reinforcement process for a behaviour</t>
+          <t>social punishment for a behaviour</t>
         </is>
       </c>
       <c r="C604" s="4" t="inlineStr">
         <is>
-          <t>A &lt;reinforcement process&gt; in which a behaviour is followed by a social event that alters the likelihood of the behaviour.</t>
+          <t xml:space="preserve">A &lt;punishment process&gt; in which the likelihood of a behaviour is increased by it being followed by a social stimulus. </t>
         </is>
       </c>
       <c r="D604" s="4" t="inlineStr">
         <is>
-          <t>reinforcement process</t>
-        </is>
-      </c>
-      <c r="E604" s="4" t="n"/>
-      <c r="F604" s="4" t="n"/>
-      <c r="G604" s="4" t="n"/>
-      <c r="H604" s="4" t="n"/>
-      <c r="I604" s="4" t="n"/>
-      <c r="J604" s="4" t="n"/>
-      <c r="K604" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L604" s="4" t="n"/>
-      <c r="M604" s="4" t="n"/>
-      <c r="N604" s="4" t="n"/>
-      <c r="O604" s="4" t="n"/>
-      <c r="P604" s="4" t="n"/>
-      <c r="Q604" s="4" t="n"/>
-      <c r="R604" s="4" t="n"/>
+          <t>punishment process</t>
+        </is>
+      </c>
+      <c r="E604" s="4" t="inlineStr"/>
+      <c r="F604" s="4" t="inlineStr"/>
+      <c r="G604" s="4" t="inlineStr"/>
+      <c r="H604" s="4" t="inlineStr"/>
+      <c r="I604" s="4" t="inlineStr"/>
+      <c r="J604" s="4" t="inlineStr"/>
+      <c r="K604" s="4" t="inlineStr"/>
+      <c r="L604" s="4" t="inlineStr"/>
+      <c r="M604" s="4" t="inlineStr"/>
+      <c r="N604" s="4" t="inlineStr"/>
+      <c r="O604" s="4" t="inlineStr"/>
+      <c r="P604" s="4" t="inlineStr"/>
+      <c r="Q604" s="4" t="inlineStr"/>
+      <c r="R604" s="4" t="inlineStr"/>
       <c r="S604" s="4" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="T604" s="4" t="n"/>
-      <c r="U604" s="4" t="n"/>
-      <c r="V604" s="4" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W604" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X604" s="4" t="n"/>
+      <c r="T604" s="4" t="inlineStr"/>
+      <c r="U604" s="4" t="inlineStr"/>
+      <c r="V604" s="4" t="inlineStr"/>
+      <c r="W604" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X604" s="4" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050779</t>
+          <t>BCIO:051042</t>
         </is>
       </c>
       <c r="B605" s="4" t="inlineStr">
         <is>
-          <t>social representation of a behaviour</t>
+          <t>social reinforcement for a behaviour</t>
         </is>
       </c>
       <c r="C605" s="4" t="inlineStr">
         <is>
-          <t>A &lt;cognitive representation&gt; about a behaviour that is shared by members of a social group.</t>
+          <t xml:space="preserve">A &lt;reinforcement process&gt; in which the likelihood of a behaviour is increased by it being followed by a social stimulus. </t>
         </is>
       </c>
       <c r="D605" s="4" t="inlineStr">
         <is>
-          <t>cognitive representation</t>
-        </is>
-      </c>
-      <c r="E605" s="4" t="n"/>
-      <c r="F605" s="4" t="n"/>
-      <c r="G605" s="4" t="inlineStr">
-        <is>
-          <t>"Social meanings" in the Social Consensus Model of Health Education</t>
-        </is>
-      </c>
-      <c r="H605" s="4" t="n"/>
-      <c r="I605" s="4" t="n"/>
-      <c r="J605" s="4" t="inlineStr">
-        <is>
-          <t>This class includes the physical representation of the behaviour and also the meanings that members of a social group assign to it.</t>
-        </is>
-      </c>
-      <c r="K605" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L605" s="4" t="n"/>
-      <c r="M605" s="4" t="n"/>
-      <c r="N605" s="4" t="n"/>
-      <c r="O605" s="4" t="n"/>
-      <c r="P605" s="4" t="n"/>
-      <c r="Q605" s="4" t="n"/>
-      <c r="R605" s="4" t="n"/>
+          <t>reinforcement process</t>
+        </is>
+      </c>
+      <c r="E605" s="4" t="inlineStr"/>
+      <c r="F605" s="4" t="inlineStr"/>
+      <c r="G605" s="4" t="inlineStr"/>
+      <c r="H605" s="4" t="inlineStr"/>
+      <c r="I605" s="4" t="inlineStr"/>
+      <c r="J605" s="4" t="inlineStr"/>
+      <c r="K605" s="4" t="inlineStr"/>
+      <c r="L605" s="4" t="inlineStr"/>
+      <c r="M605" s="4" t="inlineStr"/>
+      <c r="N605" s="4" t="inlineStr"/>
+      <c r="O605" s="4" t="inlineStr"/>
+      <c r="P605" s="4" t="inlineStr"/>
+      <c r="Q605" s="4" t="inlineStr"/>
+      <c r="R605" s="4" t="inlineStr"/>
       <c r="S605" s="4" t="inlineStr">
         <is>
           <t>Published</t>
         </is>
       </c>
-      <c r="T605" s="4" t="n"/>
-      <c r="U605" s="4" t="n"/>
-      <c r="V605" s="4" t="inlineStr">
-        <is>
-          <t>PS; JD</t>
-        </is>
-      </c>
-      <c r="W605" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X605" s="4" t="n"/>
+      <c r="T605" s="4" t="inlineStr"/>
+      <c r="U605" s="4" t="inlineStr"/>
+      <c r="V605" s="4" t="inlineStr"/>
+      <c r="W605" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X605" s="4" t="inlineStr"/>
     </row>
     <row r="606">
-      <c r="A606" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:006082</t>
-        </is>
-      </c>
-      <c r="B606" s="4" t="inlineStr">
-        <is>
-          <t>social role</t>
-        </is>
-      </c>
-      <c r="C606" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;personal role&gt; that is realised in human social processes.</t>
-        </is>
-      </c>
-      <c r="D606" s="4" t="inlineStr">
-        <is>
-          <t>personal role</t>
-        </is>
-      </c>
-      <c r="E606" s="4" t="n"/>
-      <c r="F606" s="4" t="n"/>
-      <c r="G606" s="4" t="n"/>
-      <c r="H606" s="4" t="n"/>
-      <c r="I606" s="4" t="n"/>
-      <c r="J606" s="4" t="inlineStr">
-        <is>
-          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
-        </is>
-      </c>
-      <c r="K606" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L606" s="4" t="n"/>
-      <c r="M606" s="4" t="n"/>
-      <c r="N606" s="4" t="n"/>
-      <c r="O606" s="4" t="n"/>
-      <c r="P606" s="4" t="n"/>
-      <c r="Q606" s="4" t="n"/>
-      <c r="R606" s="4" t="n"/>
-      <c r="S606" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T606" s="4" t="n"/>
-      <c r="U606" s="4" t="n"/>
-      <c r="V606" s="4" t="inlineStr">
+      <c r="A606" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050778</t>
+        </is>
+      </c>
+      <c r="B606" s="3" t="inlineStr">
+        <is>
+          <t>social reinforcement process for a behaviour</t>
+        </is>
+      </c>
+      <c r="C606" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;reinforcement process&gt; in which a behaviour is followed by a social event that alters the likelihood of the behaviour.</t>
+        </is>
+      </c>
+      <c r="D606" s="3" t="inlineStr">
+        <is>
+          <t>reinforcement process</t>
+        </is>
+      </c>
+      <c r="E606" s="3" t="n"/>
+      <c r="F606" s="3" t="n"/>
+      <c r="G606" s="3" t="n"/>
+      <c r="H606" s="3" t="n"/>
+      <c r="I606" s="3" t="n"/>
+      <c r="J606" s="3" t="n"/>
+      <c r="K606" s="3" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L606" s="3" t="n"/>
+      <c r="M606" s="3" t="n"/>
+      <c r="N606" s="3" t="n"/>
+      <c r="O606" s="3" t="n"/>
+      <c r="P606" s="3" t="n"/>
+      <c r="Q606" s="3" t="n"/>
+      <c r="R606" s="3" t="n"/>
+      <c r="S606" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="T606" s="3" t="n"/>
+      <c r="U606" s="3" t="n"/>
+      <c r="V606" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W606" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X606" s="4" t="n"/>
+      <c r="W606" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X606" s="3" t="n"/>
     </row>
     <row r="607">
       <c r="A607" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050780</t>
+          <t>BCIO:050779</t>
         </is>
       </c>
       <c r="B607" s="4" t="inlineStr">
         <is>
-          <t>social role learning</t>
+          <t>social representation of a behaviour</t>
         </is>
       </c>
       <c r="C607" s="4" t="inlineStr">
         <is>
-          <t>&lt;Learning&gt; about one’s social role.</t>
+          <t>A &lt;cognitive representation&gt; about a behaviour that is shared by members of a social group.</t>
         </is>
       </c>
       <c r="D607" s="4" t="inlineStr">
         <is>
-          <t>learning</t>
+          <t>cognitive representation</t>
         </is>
       </c>
       <c r="E607" s="4" t="n"/>
       <c r="F607" s="4" t="n"/>
       <c r="G607" s="4" t="inlineStr">
         <is>
-          <t>"Personal socialisation process" in the Systems Model of Behaviour Change</t>
+          <t>"Social meanings" in the Social Consensus Model of Health Education</t>
         </is>
       </c>
       <c r="H607" s="4" t="n"/>
       <c r="I607" s="4" t="n"/>
-      <c r="J607" s="4" t="n"/>
+      <c r="J607" s="4" t="inlineStr">
+        <is>
+          <t>This class includes the physical representation of the behaviour and also the meanings that members of a social group assign to it.</t>
+        </is>
+      </c>
       <c r="K607" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -36500,22 +36472,22 @@
     <row r="608">
       <c r="A608" s="4" t="inlineStr">
         <is>
-          <t>BCIO:006012</t>
+          <t>BCIO:006082</t>
         </is>
       </c>
       <c r="B608" s="4" t="inlineStr">
         <is>
-          <t>social skill</t>
+          <t>social role</t>
         </is>
       </c>
       <c r="C608" s="4" t="inlineStr">
         <is>
-          <t>A &lt;social behavioural capability&gt; acquired through training or practice.</t>
+          <t>A &lt;personal role&gt; that is realised in human social processes.</t>
         </is>
       </c>
       <c r="D608" s="4" t="inlineStr">
         <is>
-          <t>social behavioural capability</t>
+          <t>personal role</t>
         </is>
       </c>
       <c r="E608" s="4" t="n"/>
@@ -36523,7 +36495,11 @@
       <c r="G608" s="4" t="n"/>
       <c r="H608" s="4" t="n"/>
       <c r="I608" s="4" t="n"/>
-      <c r="J608" s="4" t="n"/>
+      <c r="J608" s="4" t="inlineStr">
+        <is>
+          <t>A role can be assigned without being realised. A person realises a role by doing something.</t>
+        </is>
+      </c>
       <c r="K608" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -36558,33 +36534,37 @@
     <row r="609">
       <c r="A609" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050441</t>
+          <t>BCIO:050780</t>
         </is>
       </c>
       <c r="B609" s="4" t="inlineStr">
         <is>
-          <t>socially-related behaviour</t>
+          <t>social role learning</t>
         </is>
       </c>
       <c r="C609" s="4" t="inlineStr">
         <is>
-          <t>An &lt;individual human behaviour&gt; that relates to the social environment.</t>
+          <t>&lt;Learning&gt; about one’s social role.</t>
         </is>
       </c>
       <c r="D609" s="4" t="inlineStr">
         <is>
-          <t>individual human behaviour</t>
+          <t>learning</t>
         </is>
       </c>
       <c r="E609" s="4" t="n"/>
       <c r="F609" s="4" t="n"/>
-      <c r="G609" s="4" t="n"/>
+      <c r="G609" s="4" t="inlineStr">
+        <is>
+          <t>"Personal socialisation process" in the Systems Model of Behaviour Change</t>
+        </is>
+      </c>
       <c r="H609" s="4" t="n"/>
       <c r="I609" s="4" t="n"/>
       <c r="J609" s="4" t="n"/>
       <c r="K609" s="4" t="inlineStr">
         <is>
-          <t>behaviour</t>
+          <t>Mechanisms of action</t>
         </is>
       </c>
       <c r="L609" s="4" t="n"/>
@@ -36603,7 +36583,7 @@
       <c r="U609" s="4" t="n"/>
       <c r="V609" s="4" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PS; JD</t>
         </is>
       </c>
       <c r="W609" s="4" t="inlineStr">
@@ -36616,22 +36596,22 @@
     <row r="610">
       <c r="A610" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050781</t>
+          <t>BCIO:006012</t>
         </is>
       </c>
       <c r="B610" s="4" t="inlineStr">
         <is>
-          <t>societal personal value</t>
+          <t>social skill</t>
         </is>
       </c>
       <c r="C610" s="4" t="inlineStr">
         <is>
-          <t>A &lt;personal value&gt; that involves regarding societal wellbeing as fundamentally important in life.</t>
+          <t>A &lt;social behavioural capability&gt; acquired through training or practice.</t>
         </is>
       </c>
       <c r="D610" s="4" t="inlineStr">
         <is>
-          <t>personal value</t>
+          <t>social behavioural capability</t>
         </is>
       </c>
       <c r="E610" s="4" t="n"/>
@@ -36674,35 +36654,35 @@
     <row r="611">
       <c r="A611" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050838</t>
+          <t>BCIO:050441</t>
         </is>
       </c>
       <c r="B611" s="4" t="inlineStr">
         <is>
-          <t>spontaneous recovery</t>
+          <t>socially-related behaviour</t>
         </is>
       </c>
       <c r="C611" s="4" t="inlineStr">
         <is>
-          <t>A &lt;bodily process&gt; in which a previously learned and then extinguished stimulus-response association becomes as least partially re-established without new pairing with a reinforcer.</t>
+          <t>An &lt;individual human behaviour&gt; that relates to the social environment.</t>
         </is>
       </c>
       <c r="D611" s="4" t="inlineStr">
         <is>
-          <t>bodily process</t>
+          <t>individual human behaviour</t>
         </is>
       </c>
       <c r="E611" s="4" t="n"/>
       <c r="F611" s="4" t="n"/>
-      <c r="G611" s="4" t="inlineStr">
-        <is>
-          <t>"Spontaneous recovery" in the Social Learning Theory</t>
-        </is>
-      </c>
+      <c r="G611" s="4" t="n"/>
       <c r="H611" s="4" t="n"/>
       <c r="I611" s="4" t="n"/>
       <c r="J611" s="4" t="n"/>
-      <c r="K611" s="4" t="n"/>
+      <c r="K611" s="4" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
       <c r="L611" s="4" t="n"/>
       <c r="M611" s="4" t="n"/>
       <c r="N611" s="4" t="n"/>
@@ -36717,40 +36697,42 @@
       </c>
       <c r="T611" s="4" t="n"/>
       <c r="U611" s="4" t="n"/>
-      <c r="V611" s="4" t="n"/>
-      <c r="W611" s="4" t="n">
-        <v>0</v>
+      <c r="V611" s="4" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W611" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="X611" s="4" t="n"/>
     </row>
     <row r="612">
       <c r="A612" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050782</t>
+          <t>BCIO:050781</t>
         </is>
       </c>
       <c r="B612" s="4" t="inlineStr">
         <is>
-          <t>stability of living conditions</t>
+          <t>societal personal value</t>
         </is>
       </c>
       <c r="C612" s="4" t="inlineStr">
         <is>
-          <t>An &lt;environmental disposition&gt; to have a stable and secure physical and social home environment.</t>
+          <t>A &lt;personal value&gt; that involves regarding societal wellbeing as fundamentally important in life.</t>
         </is>
       </c>
       <c r="D612" s="4" t="inlineStr">
         <is>
-          <t>environmental disposition</t>
+          <t>personal value</t>
         </is>
       </c>
       <c r="E612" s="4" t="n"/>
       <c r="F612" s="4" t="n"/>
-      <c r="G612" s="4" t="inlineStr">
-        <is>
-          <t>"Stable or unstable living conditions" in the Information-Motivation-Behavioural Skills Model of Adherence Behaviour</t>
-        </is>
-      </c>
+      <c r="G612" s="4" t="n"/>
       <c r="H612" s="4" t="n"/>
       <c r="I612" s="4" t="n"/>
       <c r="J612" s="4" t="n"/>
@@ -36775,7 +36757,7 @@
       <c r="U612" s="4" t="n"/>
       <c r="V612" s="4" t="inlineStr">
         <is>
-          <t>PS; JD</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="W612" s="4" t="inlineStr">
@@ -36788,43 +36770,35 @@
     <row r="613">
       <c r="A613" s="4" t="inlineStr">
         <is>
-          <t>BCIO:006072</t>
+          <t>BCIO:050838</t>
         </is>
       </c>
       <c r="B613" s="4" t="inlineStr">
         <is>
-          <t>stereotype</t>
+          <t>spontaneous recovery</t>
         </is>
       </c>
       <c r="C613" s="4" t="inlineStr">
         <is>
-          <t>A &lt;cognitive schema&gt; that when activated, guides perception, thought, emotion or behaviour toward members of a social group as having certain shared attributes, by virtue of their group membership.</t>
+          <t>A &lt;bodily process&gt; in which a previously learned and then extinguished stimulus-response association becomes as least partially re-established without new pairing with a reinforcer.</t>
         </is>
       </c>
       <c r="D613" s="4" t="inlineStr">
         <is>
-          <t>cognitive schema</t>
+          <t>bodily process</t>
         </is>
       </c>
       <c r="E613" s="4" t="n"/>
       <c r="F613" s="4" t="n"/>
       <c r="G613" s="4" t="inlineStr">
         <is>
-          <t>"Stereotypes" in the Social Consensus Model of Health Education</t>
+          <t>"Spontaneous recovery" in the Social Learning Theory</t>
         </is>
       </c>
       <c r="H613" s="4" t="n"/>
       <c r="I613" s="4" t="n"/>
-      <c r="J613" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The attributes of members are not definitional. For instance, a psychologist studying psychology is not a stereotype. </t>
-        </is>
-      </c>
-      <c r="K613" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
+      <c r="J613" s="4" t="n"/>
+      <c r="K613" s="4" t="n"/>
       <c r="L613" s="4" t="n"/>
       <c r="M613" s="4" t="n"/>
       <c r="N613" s="4" t="n"/>
@@ -36839,53 +36813,43 @@
       </c>
       <c r="T613" s="4" t="n"/>
       <c r="U613" s="4" t="n"/>
-      <c r="V613" s="4" t="inlineStr">
-        <is>
-          <t>PS; JD</t>
-        </is>
-      </c>
-      <c r="W613" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="V613" s="4" t="n"/>
+      <c r="W613" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="X613" s="4" t="n"/>
     </row>
     <row r="614">
       <c r="A614" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050783</t>
+          <t>BCIO:050782</t>
         </is>
       </c>
       <c r="B614" s="4" t="inlineStr">
         <is>
-          <t>stimulus</t>
+          <t>stability of living conditions</t>
         </is>
       </c>
       <c r="C614" s="4" t="inlineStr">
         <is>
-          <t>An &lt;entity&gt; that acts as an input to a perceptual process leading to a thought, feeling or action.</t>
+          <t>An &lt;environmental disposition&gt; to have a stable and secure physical and social home environment.</t>
         </is>
       </c>
       <c r="D614" s="4" t="inlineStr">
         <is>
-          <t>entity</t>
+          <t>environmental disposition</t>
         </is>
       </c>
       <c r="E614" s="4" t="n"/>
       <c r="F614" s="4" t="n"/>
       <c r="G614" s="4" t="inlineStr">
         <is>
-          <t>a loud noise, the sight of a treadmill, the picture of specific foods</t>
+          <t>"Stable or unstable living conditions" in the Information-Motivation-Behavioural Skills Model of Adherence Behaviour</t>
         </is>
       </c>
       <c r="H614" s="4" t="n"/>
       <c r="I614" s="4" t="n"/>
-      <c r="J614" s="4" t="inlineStr">
-        <is>
-          <t>A stimulus can be naturally occurring or used as component of Behaviour Change Techniques (BCTs). These are part of learning processes and operationalized as part of BCTs.</t>
-        </is>
-      </c>
+      <c r="J614" s="4" t="n"/>
       <c r="K614" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -36907,7 +36871,7 @@
       <c r="U614" s="4" t="n"/>
       <c r="V614" s="4" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PS; JD</t>
         </is>
       </c>
       <c r="W614" s="4" t="inlineStr">
@@ -36920,36 +36884,36 @@
     <row r="615">
       <c r="A615" s="4" t="inlineStr">
         <is>
-          <t>BCIO:006124</t>
+          <t>BCIO:006072</t>
         </is>
       </c>
       <c r="B615" s="4" t="inlineStr">
         <is>
-          <t>stimulus generalisation in learning</t>
+          <t>stereotype</t>
         </is>
       </c>
       <c r="C615" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;Generalisation in learning&gt; concerning the antecedent stimulus. </t>
+          <t>A &lt;cognitive schema&gt; that when activated, guides perception, thought, emotion or behaviour toward members of a social group as having certain shared attributes, by virtue of their group membership.</t>
         </is>
       </c>
       <c r="D615" s="4" t="inlineStr">
         <is>
-          <t>generalisation in learning</t>
+          <t>cognitive schema</t>
         </is>
       </c>
       <c r="E615" s="4" t="n"/>
       <c r="F615" s="4" t="n"/>
       <c r="G615" s="4" t="inlineStr">
         <is>
-          <t>"Generalisation" in the Social Learning Theory</t>
+          <t>"Stereotypes" in the Social Consensus Model of Health Education</t>
         </is>
       </c>
       <c r="H615" s="4" t="n"/>
       <c r="I615" s="4" t="n"/>
       <c r="J615" s="4" t="inlineStr">
         <is>
-          <t>The label 'Generalisation of target  behavior' is used for a behaviour change technique (BCT) in the BCT Taxonomy v1 (Michie et al., 2013). The definition for this BCT reads as follows: 'Advise to perform the wanted behaviour,  which is already performed in a particular situation, in another situation.' Therefore, the BCT is the advice to perform the behaviour, whereas the MoA is a learning process that occurs in the brain.</t>
+          <t xml:space="preserve">The attributes of members are not definitional. For instance, a psychologist studying psychology is not a stereotype. </t>
         </is>
       </c>
       <c r="K615" s="4" t="inlineStr">
@@ -36973,7 +36937,7 @@
       <c r="U615" s="4" t="n"/>
       <c r="V615" s="4" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PS; JD</t>
         </is>
       </c>
       <c r="W615" s="4" t="inlineStr">
@@ -36986,36 +36950,36 @@
     <row r="616">
       <c r="A616" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050784</t>
+          <t>BCIO:050783</t>
         </is>
       </c>
       <c r="B616" s="4" t="inlineStr">
         <is>
-          <t>stimulus-impulse association</t>
+          <t>stimulus</t>
         </is>
       </c>
       <c r="C616" s="4" t="inlineStr">
         <is>
-          <t>A &lt;mental process&gt; in which a stimulus strengthens a tendency for an impulse.</t>
+          <t>An &lt;entity&gt; that acts as an input to a perceptual process leading to a thought, feeling or action.</t>
         </is>
       </c>
       <c r="D616" s="4" t="inlineStr">
         <is>
-          <t>mental process</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="E616" s="4" t="n"/>
       <c r="F616" s="4" t="n"/>
       <c r="G616" s="4" t="inlineStr">
         <is>
-          <t>"Impulsive system" in the Reflective Impulsive Model</t>
+          <t>a loud noise, the sight of a treadmill, the picture of specific foods</t>
         </is>
       </c>
       <c r="H616" s="4" t="n"/>
       <c r="I616" s="4" t="n"/>
       <c r="J616" s="4" t="inlineStr">
         <is>
-          <t>Stimulus-impulse association is part of operant learning processes.</t>
+          <t>A stimulus can be naturally occurring or used as component of Behaviour Change Techniques (BCTs). These are part of learning processes and operationalized as part of BCTs.</t>
         </is>
       </c>
       <c r="K616" s="4" t="inlineStr">
@@ -37039,7 +37003,7 @@
       <c r="U616" s="4" t="n"/>
       <c r="V616" s="4" t="inlineStr">
         <is>
-          <t>PS; JD</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="W616" s="4" t="inlineStr">
@@ -37052,36 +37016,36 @@
     <row r="617">
       <c r="A617" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050785</t>
+          <t>BCIO:006124</t>
         </is>
       </c>
       <c r="B617" s="4" t="inlineStr">
         <is>
-          <t>strength of attention</t>
+          <t>stimulus generalisation in learning</t>
         </is>
       </c>
       <c r="C617" s="4" t="inlineStr">
         <is>
-          <t>A &lt;mental process attribute&gt; that is the extent to which attentional resources are focused on a target.</t>
+          <t xml:space="preserve">&lt;Generalisation in learning&gt; concerning the antecedent stimulus. </t>
         </is>
       </c>
       <c r="D617" s="4" t="inlineStr">
         <is>
-          <t>mental process attribute</t>
+          <t>generalisation in learning</t>
         </is>
       </c>
       <c r="E617" s="4" t="n"/>
       <c r="F617" s="4" t="n"/>
       <c r="G617" s="4" t="inlineStr">
         <is>
-          <t>"Strength of engagement / motivation" in the Regulatory Fit Theory</t>
+          <t>"Generalisation" in the Social Learning Theory</t>
         </is>
       </c>
       <c r="H617" s="4" t="n"/>
       <c r="I617" s="4" t="n"/>
       <c r="J617" s="4" t="inlineStr">
         <is>
-          <t>Target refers to anything that can be attended to, whether it be an object, an attribute of an object, information or a process.</t>
+          <t>The label 'Generalisation of target  behavior' is used for a behaviour change technique (BCT) in the BCT Taxonomy v1 (Michie et al., 2013). The definition for this BCT reads as follows: 'Advise to perform the wanted behaviour,  which is already performed in a particular situation, in another situation.' Therefore, the BCT is the advice to perform the behaviour, whereas the MoA is a learning process that occurs in the brain.</t>
         </is>
       </c>
       <c r="K617" s="4" t="inlineStr">
@@ -37105,7 +37069,7 @@
       <c r="U617" s="4" t="n"/>
       <c r="V617" s="4" t="inlineStr">
         <is>
-          <t>PS; JD</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="W617" s="4" t="inlineStr">
@@ -37118,34 +37082,38 @@
     <row r="618">
       <c r="A618" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050883</t>
+          <t>BCIO:050784</t>
         </is>
       </c>
       <c r="B618" s="4" t="inlineStr">
         <is>
-          <t>strength of group support for an intervention</t>
+          <t>stimulus-impulse association</t>
         </is>
       </c>
       <c r="C618" s="4" t="inlineStr">
         <is>
-          <t>A &lt;social group attribute&gt; that is the extent to which its members positively evaluate an intervention.</t>
+          <t>A &lt;mental process&gt; in which a stimulus strengthens a tendency for an impulse.</t>
         </is>
       </c>
       <c r="D618" s="4" t="inlineStr">
         <is>
-          <t>social group attribute</t>
+          <t>mental process</t>
         </is>
       </c>
       <c r="E618" s="4" t="n"/>
       <c r="F618" s="4" t="n"/>
       <c r="G618" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Community priorities" in the Social Ecological Model of Behaviour Change </t>
+          <t>"Impulsive system" in the Reflective Impulsive Model</t>
         </is>
       </c>
       <c r="H618" s="4" t="n"/>
       <c r="I618" s="4" t="n"/>
-      <c r="J618" s="4" t="n"/>
+      <c r="J618" s="4" t="inlineStr">
+        <is>
+          <t>Stimulus-impulse association is part of operant learning processes.</t>
+        </is>
+      </c>
       <c r="K618" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -37178,275 +37146,279 @@
       <c r="X618" s="4" t="n"/>
     </row>
     <row r="619">
-      <c r="A619" t="inlineStr">
+      <c r="A619" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050785</t>
+        </is>
+      </c>
+      <c r="B619" s="4" t="inlineStr">
+        <is>
+          <t>strength of attention</t>
+        </is>
+      </c>
+      <c r="C619" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;mental process attribute&gt; that is the extent to which attentional resources are focused on a target.</t>
+        </is>
+      </c>
+      <c r="D619" s="4" t="inlineStr">
+        <is>
+          <t>mental process attribute</t>
+        </is>
+      </c>
+      <c r="E619" s="4" t="n"/>
+      <c r="F619" s="4" t="n"/>
+      <c r="G619" s="4" t="inlineStr">
+        <is>
+          <t>"Strength of engagement / motivation" in the Regulatory Fit Theory</t>
+        </is>
+      </c>
+      <c r="H619" s="4" t="n"/>
+      <c r="I619" s="4" t="n"/>
+      <c r="J619" s="4" t="inlineStr">
+        <is>
+          <t>Target refers to anything that can be attended to, whether it be an object, an attribute of an object, information or a process.</t>
+        </is>
+      </c>
+      <c r="K619" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L619" s="4" t="n"/>
+      <c r="M619" s="4" t="n"/>
+      <c r="N619" s="4" t="n"/>
+      <c r="O619" s="4" t="n"/>
+      <c r="P619" s="4" t="n"/>
+      <c r="Q619" s="4" t="n"/>
+      <c r="R619" s="4" t="n"/>
+      <c r="S619" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T619" s="4" t="n"/>
+      <c r="U619" s="4" t="n"/>
+      <c r="V619" s="4" t="inlineStr">
+        <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W619" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X619" s="4" t="n"/>
+    </row>
+    <row r="620">
+      <c r="A620" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050883</t>
+        </is>
+      </c>
+      <c r="B620" s="4" t="inlineStr">
+        <is>
+          <t>strength of group support for an intervention</t>
+        </is>
+      </c>
+      <c r="C620" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;social group attribute&gt; that is the extent to which its members positively evaluate an intervention.</t>
+        </is>
+      </c>
+      <c r="D620" s="4" t="inlineStr">
+        <is>
+          <t>social group attribute</t>
+        </is>
+      </c>
+      <c r="E620" s="4" t="n"/>
+      <c r="F620" s="4" t="n"/>
+      <c r="G620" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">"Community priorities" in the Social Ecological Model of Behaviour Change </t>
+        </is>
+      </c>
+      <c r="H620" s="4" t="n"/>
+      <c r="I620" s="4" t="n"/>
+      <c r="J620" s="4" t="n"/>
+      <c r="K620" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L620" s="4" t="n"/>
+      <c r="M620" s="4" t="n"/>
+      <c r="N620" s="4" t="n"/>
+      <c r="O620" s="4" t="n"/>
+      <c r="P620" s="4" t="n"/>
+      <c r="Q620" s="4" t="n"/>
+      <c r="R620" s="4" t="n"/>
+      <c r="S620" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T620" s="4" t="n"/>
+      <c r="U620" s="4" t="n"/>
+      <c r="V620" s="4" t="inlineStr">
+        <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W620" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X620" s="4" t="n"/>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
         <is>
           <t xml:space="preserve">MFOEM:000006 </t>
         </is>
       </c>
-      <c r="B619" t="inlineStr">
+      <c r="B621" t="inlineStr">
         <is>
           <t>subjective affective feeling</t>
         </is>
       </c>
-      <c r="C619" t="inlineStr">
+      <c r="C621" t="inlineStr">
         <is>
           <t>An &lt;affective process&gt; that involves the experience of internal or external sensory stimuli.</t>
         </is>
       </c>
-      <c r="D619" t="inlineStr">
+      <c r="D621" t="inlineStr">
         <is>
           <t>affective process</t>
         </is>
       </c>
-      <c r="F619" t="inlineStr">
+      <c r="F621" t="inlineStr">
         <is>
           <t>The conscious experience that a person has of feelings in their body (e.g., hunger), their mood (e.g., feeling cheerful) and their emotion (e.g., feeling nervous), in response to internal or external stimuli.</t>
         </is>
       </c>
-      <c r="G619" t="inlineStr">
+      <c r="G621" t="inlineStr">
         <is>
           <t>"Wants" in the PRIME theory; "Regulatory fit" in the Regulatory Fit Theory</t>
         </is>
       </c>
-      <c r="I619" t="inlineStr">
+      <c r="I621" t="inlineStr">
         <is>
           <t>Feeling calm; hunger; pain</t>
         </is>
       </c>
-      <c r="J619" t="inlineStr">
+      <c r="J621" t="inlineStr">
         <is>
           <t>'Subjective affective feeling can have greater or weaker physiological or mental components. The bodily process that are experienced will usually involve some mental process.
 Bodily sensation and the experiences of emotions (e.g., feeling calm) would both qualify as examples of 'subjective affective feeling'.
 As a subclass of 'affective process', subjective affective feelings have valence. Valence refers to the 'the subjective value of an event, object, person, or other entity in the life space of the individual' (https://dictionary.apa.org/valence). Valence ranges from negative to positive.</t>
         </is>
       </c>
-      <c r="K619" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S619" t="inlineStr">
+      <c r="K621" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S621" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V619" t="inlineStr">
+      <c r="V621" t="inlineStr">
         <is>
           <t>PS; JD</t>
         </is>
       </c>
-      <c r="W619" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="620">
-      <c r="A620" t="inlineStr">
+      <c r="W621" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
         <is>
           <t>ADDICTO:0000511</t>
         </is>
       </c>
-      <c r="B620" t="inlineStr">
+      <c r="B622" t="inlineStr">
         <is>
           <t>subjective craving</t>
         </is>
       </c>
-      <c r="C620" t="inlineStr">
+      <c r="C622" t="inlineStr">
         <is>
           <t>A &lt;subjective affective feeling&gt; involving a strong desire or urge.</t>
         </is>
       </c>
-      <c r="D620" t="inlineStr">
+      <c r="D622" t="inlineStr">
         <is>
           <t>subjective affective feeling</t>
         </is>
       </c>
-      <c r="K620" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S620" t="inlineStr">
+      <c r="K622" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S622" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="U620" t="inlineStr">
+      <c r="U622" t="inlineStr">
         <is>
           <t>RW: I've made the edits I suggest pending agreement from the rest of the team 23 Feb 22</t>
         </is>
       </c>
-      <c r="V620" t="inlineStr">
+      <c r="V622" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W620" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="621">
-      <c r="A621" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050323</t>
-        </is>
-      </c>
-      <c r="B621" s="4" t="inlineStr">
-        <is>
-          <t>subjective feeling</t>
-        </is>
-      </c>
-      <c r="C621" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;mental process&gt; that involves the experience of internal or external sensory stimuli.</t>
-        </is>
-      </c>
-      <c r="D621" s="4" t="inlineStr">
-        <is>
-          <t>mental process</t>
-        </is>
-      </c>
-      <c r="E621" s="4" t="n"/>
-      <c r="F621" s="4" t="n"/>
-      <c r="G621" s="4" t="inlineStr">
-        <is>
-          <t>Feeling ticklish, feeling tingling</t>
-        </is>
-      </c>
-      <c r="H621" s="4" t="n"/>
-      <c r="I621" s="4" t="n"/>
-      <c r="J621" s="4" t="inlineStr">
-        <is>
-          <t>If a subjective feeling is valenced (i.e., an affective process), the more granular class “subjective affective feeling” can be used to capture this feeling.</t>
-        </is>
-      </c>
-      <c r="K621" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L621" s="4" t="n"/>
-      <c r="M621" s="4" t="n"/>
-      <c r="N621" s="4" t="n"/>
-      <c r="O621" s="4" t="n"/>
-      <c r="P621" s="4" t="n"/>
-      <c r="Q621" s="4" t="n"/>
-      <c r="R621" s="4" t="n"/>
-      <c r="S621" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T621" s="4" t="n"/>
-      <c r="U621" s="4" t="n"/>
-      <c r="V621" s="4" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W621" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X621" s="4" t="n"/>
-    </row>
-    <row r="622">
-      <c r="A622" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050316</t>
-        </is>
-      </c>
-      <c r="B622" s="4" t="inlineStr">
-        <is>
-          <t>subjective need</t>
-        </is>
-      </c>
-      <c r="C622" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;subjective affective feeling&gt; that is an attraction to an imagined scenario involving anticipated relief from or avoidance of mental or physical discomfort.</t>
-        </is>
-      </c>
-      <c r="D622" s="4" t="inlineStr">
-        <is>
-          <t>subjective affective feeling</t>
-        </is>
-      </c>
-      <c r="E622" s="4" t="n"/>
-      <c r="F622" s="4" t="inlineStr">
-        <is>
-          <t>A feeling of anticipated relief or avoidance of discomfort.</t>
-        </is>
-      </c>
-      <c r="G622" s="4" t="n"/>
-      <c r="H622" s="4" t="n"/>
-      <c r="I622" s="4" t="n"/>
-      <c r="J622" s="4" t="n"/>
-      <c r="K622" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L622" s="4" t="n"/>
-      <c r="M622" s="4" t="n"/>
-      <c r="N622" s="4" t="n"/>
-      <c r="O622" s="4" t="n"/>
-      <c r="P622" s="4" t="n"/>
-      <c r="Q622" s="4" t="n"/>
-      <c r="R622" s="4" t="n"/>
-      <c r="S622" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T622" s="4" t="n"/>
-      <c r="U622" s="4" t="n"/>
-      <c r="V622" s="4" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W622" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X622" s="4" t="n"/>
+      <c r="W622" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="623">
       <c r="A623" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050317</t>
+          <t>BCIO:050323</t>
         </is>
       </c>
       <c r="B623" s="4" t="inlineStr">
         <is>
-          <t>subjective want</t>
+          <t>subjective feeling</t>
         </is>
       </c>
       <c r="C623" s="4" t="inlineStr">
         <is>
-          <t>A &lt;subjective affective feeling&gt; that is an attraction to an imagined scenario involving anticipated pleasure or satisfaction.</t>
+          <t>A &lt;mental process&gt; that involves the experience of internal or external sensory stimuli.</t>
         </is>
       </c>
       <c r="D623" s="4" t="inlineStr">
         <is>
-          <t>subjective affective feeling</t>
+          <t>mental process</t>
         </is>
       </c>
       <c r="E623" s="4" t="n"/>
       <c r="F623" s="4" t="n"/>
       <c r="G623" s="4" t="inlineStr">
         <is>
-          <t>"Value from worth" in the Regulatory Fit Theory</t>
+          <t>Feeling ticklish, feeling tingling</t>
         </is>
       </c>
       <c r="H623" s="4" t="n"/>
       <c r="I623" s="4" t="n"/>
-      <c r="J623" s="4" t="n"/>
+      <c r="J623" s="4" t="inlineStr">
+        <is>
+          <t>If a subjective feeling is valenced (i.e., an affective process), the more granular class “subjective affective feeling” can be used to capture this feeling.</t>
+        </is>
+      </c>
       <c r="K623" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -37479,290 +37451,315 @@
       <c r="X623" s="4" t="n"/>
     </row>
     <row r="624">
-      <c r="A624" t="inlineStr">
+      <c r="A624" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050316</t>
+        </is>
+      </c>
+      <c r="B624" s="4" t="inlineStr">
+        <is>
+          <t>subjective need</t>
+        </is>
+      </c>
+      <c r="C624" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;subjective affective feeling&gt; that is an attraction to an imagined scenario involving anticipated relief from or avoidance of mental or physical discomfort.</t>
+        </is>
+      </c>
+      <c r="D624" s="4" t="inlineStr">
+        <is>
+          <t>subjective affective feeling</t>
+        </is>
+      </c>
+      <c r="E624" s="4" t="n"/>
+      <c r="F624" s="4" t="inlineStr">
+        <is>
+          <t>A feeling of anticipated relief or avoidance of discomfort.</t>
+        </is>
+      </c>
+      <c r="G624" s="4" t="n"/>
+      <c r="H624" s="4" t="n"/>
+      <c r="I624" s="4" t="n"/>
+      <c r="J624" s="4" t="n"/>
+      <c r="K624" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L624" s="4" t="n"/>
+      <c r="M624" s="4" t="n"/>
+      <c r="N624" s="4" t="n"/>
+      <c r="O624" s="4" t="n"/>
+      <c r="P624" s="4" t="n"/>
+      <c r="Q624" s="4" t="n"/>
+      <c r="R624" s="4" t="n"/>
+      <c r="S624" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T624" s="4" t="n"/>
+      <c r="U624" s="4" t="n"/>
+      <c r="V624" s="4" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W624" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X624" s="4" t="n"/>
+    </row>
+    <row r="625">
+      <c r="A625" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050317</t>
+        </is>
+      </c>
+      <c r="B625" s="4" t="inlineStr">
+        <is>
+          <t>subjective want</t>
+        </is>
+      </c>
+      <c r="C625" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;subjective affective feeling&gt; that is an attraction to an imagined scenario involving anticipated pleasure or satisfaction.</t>
+        </is>
+      </c>
+      <c r="D625" s="4" t="inlineStr">
+        <is>
+          <t>subjective affective feeling</t>
+        </is>
+      </c>
+      <c r="E625" s="4" t="n"/>
+      <c r="F625" s="4" t="n"/>
+      <c r="G625" s="4" t="inlineStr">
+        <is>
+          <t>"Value from worth" in the Regulatory Fit Theory</t>
+        </is>
+      </c>
+      <c r="H625" s="4" t="n"/>
+      <c r="I625" s="4" t="n"/>
+      <c r="J625" s="4" t="n"/>
+      <c r="K625" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L625" s="4" t="n"/>
+      <c r="M625" s="4" t="n"/>
+      <c r="N625" s="4" t="n"/>
+      <c r="O625" s="4" t="n"/>
+      <c r="P625" s="4" t="n"/>
+      <c r="Q625" s="4" t="n"/>
+      <c r="R625" s="4" t="n"/>
+      <c r="S625" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T625" s="4" t="n"/>
+      <c r="U625" s="4" t="n"/>
+      <c r="V625" s="4" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W625" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X625" s="4" t="n"/>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
         <is>
           <t xml:space="preserve">MF:0000088 </t>
         </is>
       </c>
-      <c r="B624" t="inlineStr">
+      <c r="B626" t="inlineStr">
         <is>
           <t>subliminal process</t>
         </is>
       </c>
-      <c r="C624" t="inlineStr">
+      <c r="C626" t="inlineStr">
         <is>
           <t>A &lt;mental process&gt; that involves neuronal activity in response to a sensory stimulus but which is not the subject of consciousness.</t>
         </is>
       </c>
-      <c r="D624" t="inlineStr">
+      <c r="D626" t="inlineStr">
         <is>
           <t>mental process</t>
         </is>
       </c>
-      <c r="K624" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S624" t="inlineStr">
+      <c r="K626" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S626" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V624" t="inlineStr">
+      <c r="V626" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W624" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="625">
-      <c r="A625" t="inlineStr">
+      <c r="W626" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
         <is>
           <t>ADDICTO:0001212</t>
         </is>
       </c>
-      <c r="B625" t="inlineStr">
+      <c r="B627" t="inlineStr">
         <is>
           <t>substance dependence</t>
         </is>
       </c>
-      <c r="C625" t="inlineStr">
+      <c r="C627" t="inlineStr">
         <is>
           <t>A &lt;bodily disposition&gt; which is realised as impaired functioning following reduction or termination of use of a psychoactive substance.</t>
         </is>
       </c>
-      <c r="D625" t="inlineStr">
+      <c r="D627" t="inlineStr">
         <is>
           <t>bodily disposition</t>
         </is>
       </c>
-      <c r="J625" t="inlineStr">
+      <c r="J627" t="inlineStr">
         <is>
           <t>While 'addiction' is a disposition relating to experience motivation to use a substance, 'substance dependence' refers to 'disposition related to the impaired functioning in the absence of a substance'.</t>
         </is>
       </c>
-      <c r="K625" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S625" t="inlineStr">
+      <c r="K627" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S627" t="inlineStr">
         <is>
           <t>External</t>
         </is>
       </c>
-      <c r="V625" t="inlineStr">
+      <c r="V627" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W625" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-    </row>
-    <row r="626">
-      <c r="A626" s="4" t="inlineStr">
+      <c r="W627" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="4" t="inlineStr">
         <is>
           <t>BCIO:050786</t>
         </is>
       </c>
-      <c r="B626" s="4" t="inlineStr">
+      <c r="B628" s="4" t="inlineStr">
         <is>
           <t>supportive social environmental disposition</t>
         </is>
       </c>
-      <c r="C626" s="4" t="inlineStr">
+      <c r="C628" s="4" t="inlineStr">
         <is>
           <t>A &lt;social environmental disposition&gt; that is the extend to which the social environemental system benefits the person’s thoughts, emotions or behaviours.</t>
         </is>
       </c>
-      <c r="D626" s="4" t="inlineStr">
+      <c r="D628" s="4" t="inlineStr">
         <is>
           <t>social environmental disposition</t>
         </is>
       </c>
-      <c r="E626" s="4" t="n"/>
-      <c r="F626" s="4" t="n"/>
-      <c r="G626" s="4" t="n"/>
-      <c r="H626" s="4" t="n"/>
-      <c r="I626" s="4" t="n"/>
-      <c r="J626" s="4" t="inlineStr">
+      <c r="E628" s="4" t="n"/>
+      <c r="F628" s="4" t="n"/>
+      <c r="G628" s="4" t="n"/>
+      <c r="H628" s="4" t="n"/>
+      <c r="I628" s="4" t="n"/>
+      <c r="J628" s="4" t="inlineStr">
         <is>
           <t>If you are interested in capturing a social environmental system that is supportive rather than to what extend a system is supportive, then please refer to "supportive social environmental system".</t>
         </is>
       </c>
-      <c r="K626" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L626" s="4" t="n"/>
-      <c r="M626" s="4" t="n"/>
-      <c r="N626" s="4" t="n"/>
-      <c r="O626" s="4" t="n"/>
-      <c r="P626" s="4" t="n"/>
-      <c r="Q626" s="4" t="n"/>
-      <c r="R626" s="4" t="n"/>
-      <c r="S626" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T626" s="4" t="n"/>
-      <c r="U626" s="4" t="n"/>
-      <c r="V626" s="4" t="inlineStr">
+      <c r="K628" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L628" s="4" t="n"/>
+      <c r="M628" s="4" t="n"/>
+      <c r="N628" s="4" t="n"/>
+      <c r="O628" s="4" t="n"/>
+      <c r="P628" s="4" t="n"/>
+      <c r="Q628" s="4" t="n"/>
+      <c r="R628" s="4" t="n"/>
+      <c r="S628" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T628" s="4" t="n"/>
+      <c r="U628" s="4" t="n"/>
+      <c r="V628" s="4" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W626" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X626" s="4" t="n"/>
-    </row>
-    <row r="627">
-      <c r="A627" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050787</t>
-        </is>
-      </c>
-      <c r="B627" s="4" t="inlineStr">
-        <is>
-          <t>supportive social environmental system</t>
-        </is>
-      </c>
-      <c r="C627" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;social environmental system&gt; that benefits the person’s thoughts, emotions or behaviours.</t>
-        </is>
-      </c>
-      <c r="D627" s="4" t="inlineStr">
-        <is>
-          <t>social environmental system</t>
-        </is>
-      </c>
-      <c r="E627" s="4" t="n"/>
-      <c r="F627" s="4" t="n"/>
-      <c r="G627" s="4" t="inlineStr">
-        <is>
-          <t>"Supportive Environment" in the Integrated Theoretical Model for Alcohol and Other Drug Abuse Prevention; "Organisational support" in the Social Ecological Model of Behaviour Change</t>
-        </is>
-      </c>
-      <c r="H627" s="4" t="n"/>
-      <c r="I627" s="4" t="n"/>
-      <c r="J627" s="4" t="inlineStr">
-        <is>
-          <t>If you are interested in capturing to what extend a system is supportive rather than the system itself, then please refer to "supportive social environmental disposition".</t>
-        </is>
-      </c>
-      <c r="K627" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L627" s="4" t="n"/>
-      <c r="M627" s="4" t="n"/>
-      <c r="N627" s="4" t="n"/>
-      <c r="O627" s="4" t="n"/>
-      <c r="P627" s="4" t="n"/>
-      <c r="Q627" s="4" t="n"/>
-      <c r="R627" s="4" t="n"/>
-      <c r="S627" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T627" s="4" t="n"/>
-      <c r="U627" s="4" t="n"/>
-      <c r="V627" s="4" t="inlineStr">
-        <is>
-          <t>PS; JD</t>
-        </is>
-      </c>
-      <c r="W627" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X627" s="4" t="n"/>
-    </row>
-    <row r="628">
-      <c r="A628" t="inlineStr">
-        <is>
-          <t>MFOEM:000032</t>
-        </is>
-      </c>
-      <c r="B628" t="inlineStr">
-        <is>
-          <t>surprise</t>
-        </is>
-      </c>
-      <c r="C628" t="inlineStr">
-        <is>
-          <t xml:space="preserve">An emotion caused by encountering unexpected events. </t>
-        </is>
-      </c>
-      <c r="D628" t="inlineStr">
-        <is>
-          <t>emotion process</t>
-        </is>
-      </c>
-      <c r="K628" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S628" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="W628" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="W628" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X628" s="4" t="n"/>
     </row>
     <row r="629">
       <c r="A629" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050788</t>
+          <t>BCIO:050787</t>
         </is>
       </c>
       <c r="B629" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">symbol processing skill </t>
+          <t>supportive social environmental system</t>
         </is>
       </c>
       <c r="C629" s="4" t="inlineStr">
         <is>
-          <t>A &lt;mental skill&gt; to be able to process information in the form of symbols.</t>
+          <t>A &lt;social environmental system&gt; that benefits the person’s thoughts, emotions or behaviours.</t>
         </is>
       </c>
       <c r="D629" s="4" t="inlineStr">
         <is>
-          <t>mental skill</t>
+          <t>social environmental system</t>
         </is>
       </c>
       <c r="E629" s="4" t="n"/>
       <c r="F629" s="4" t="n"/>
       <c r="G629" s="4" t="inlineStr">
         <is>
-          <t>"Symbolising capability" in the Social Cognitive Theory</t>
+          <t>"Supportive Environment" in the Integrated Theoretical Model for Alcohol and Other Drug Abuse Prevention; "Organisational support" in the Social Ecological Model of Behaviour Change</t>
         </is>
       </c>
       <c r="H629" s="4" t="n"/>
       <c r="I629" s="4" t="n"/>
-      <c r="J629" s="4" t="n"/>
+      <c r="J629" s="4" t="inlineStr">
+        <is>
+          <t>If you are interested in capturing to what extend a system is supportive rather than the system itself, then please refer to "supportive social environmental disposition".</t>
+        </is>
+      </c>
       <c r="K629" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -37797,22 +37794,22 @@
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>RO:0002577</t>
+          <t>MFOEM:000032</t>
         </is>
       </c>
       <c r="B630" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>surprise</t>
         </is>
       </c>
       <c r="C630" t="inlineStr">
         <is>
-          <t>A &lt;material entity&gt; consisting of multiple components that are causally integrated.</t>
+          <t xml:space="preserve">An emotion caused by encountering unexpected events. </t>
         </is>
       </c>
       <c r="D630" t="inlineStr">
         <is>
-          <t>material entity</t>
+          <t>emotion process</t>
         </is>
       </c>
       <c r="K630" t="inlineStr">
@@ -37823,11 +37820,6 @@
       <c r="S630" t="inlineStr">
         <is>
           <t>External</t>
-        </is>
-      </c>
-      <c r="V630" t="inlineStr">
-        <is>
-          <t>PS</t>
         </is>
       </c>
       <c r="W630" t="inlineStr">
@@ -37839,33 +37831,33 @@
     <row r="631">
       <c r="A631" s="4" t="inlineStr">
         <is>
-          <t>BCIO:006163</t>
+          <t>BCIO:050788</t>
         </is>
       </c>
       <c r="B631" s="4" t="inlineStr">
         <is>
-          <t>targeted mental distancing</t>
+          <t xml:space="preserve">symbol processing skill </t>
         </is>
       </c>
       <c r="C631" s="4" t="inlineStr">
         <is>
-          <t>&lt;Mental distancing&gt; that involves identifying particular immediate thoughts and intentionally detaching from these thoughts.</t>
+          <t>A &lt;mental skill&gt; to be able to process information in the form of symbols.</t>
         </is>
       </c>
       <c r="D631" s="4" t="inlineStr">
         <is>
-          <t>mental distancing</t>
+          <t>mental skill</t>
         </is>
       </c>
       <c r="E631" s="4" t="n"/>
       <c r="F631" s="4" t="n"/>
-      <c r="G631" s="4" t="n"/>
+      <c r="G631" s="4" t="inlineStr">
+        <is>
+          <t>"Symbolising capability" in the Social Cognitive Theory</t>
+        </is>
+      </c>
       <c r="H631" s="4" t="n"/>
-      <c r="I631" s="4" t="inlineStr">
-        <is>
-          <t>targeted decentring</t>
-        </is>
-      </c>
+      <c r="I631" s="4" t="n"/>
       <c r="J631" s="4" t="n"/>
       <c r="K631" s="4" t="inlineStr">
         <is>
@@ -37888,112 +37880,88 @@
       <c r="U631" s="4" t="n"/>
       <c r="V631" s="4" t="inlineStr">
         <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W631" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X631" s="4" t="n"/>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>RO:0002577</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>A &lt;material entity&gt; consisting of multiple components that are causally integrated.</t>
+        </is>
+      </c>
+      <c r="D632" t="inlineStr">
+        <is>
+          <t>material entity</t>
+        </is>
+      </c>
+      <c r="K632" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S632" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V632" t="inlineStr">
+        <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W631" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X631" s="4" t="n"/>
-    </row>
-    <row r="632">
-      <c r="A632" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050789</t>
-        </is>
-      </c>
-      <c r="B632" s="4" t="inlineStr">
-        <is>
-          <t>technology availability</t>
-        </is>
-      </c>
-      <c r="C632" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;behavioural opportunity&gt; that involves the extend to which technology is available in the environmental system.</t>
-        </is>
-      </c>
-      <c r="D632" s="4" t="inlineStr">
-        <is>
-          <t>behavioural opportunity</t>
-        </is>
-      </c>
-      <c r="E632" s="4" t="n"/>
-      <c r="F632" s="4" t="n"/>
-      <c r="G632" s="4" t="inlineStr">
-        <is>
-          <t>"Technology" in the Needs-Opportunity-Abilities Model</t>
-        </is>
-      </c>
-      <c r="H632" s="4" t="n"/>
-      <c r="I632" s="4" t="n"/>
-      <c r="J632" s="4" t="n"/>
-      <c r="K632" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L632" s="4" t="n"/>
-      <c r="M632" s="4" t="n"/>
-      <c r="N632" s="4" t="n"/>
-      <c r="O632" s="4" t="n"/>
-      <c r="P632" s="4" t="n"/>
-      <c r="Q632" s="4" t="n"/>
-      <c r="R632" s="4" t="n"/>
-      <c r="S632" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T632" s="4" t="n"/>
-      <c r="U632" s="4" t="n"/>
-      <c r="V632" s="4" t="inlineStr">
-        <is>
-          <t>PS; JD</t>
-        </is>
-      </c>
-      <c r="W632" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X632" s="4" t="n"/>
+      <c r="W632" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="633">
       <c r="A633" s="4" t="inlineStr">
         <is>
-          <t>BCIO:006091</t>
+          <t>BCIO:006163</t>
         </is>
       </c>
       <c r="B633" s="4" t="inlineStr">
         <is>
-          <t>temporal behavioural opportunity</t>
+          <t>targeted mental distancing</t>
         </is>
       </c>
       <c r="C633" s="4" t="inlineStr">
         <is>
-          <t>A &lt;physical behavioural opportunity&gt; that involves the person having sufficient time or a suitable period.</t>
+          <t>&lt;Mental distancing&gt; that involves identifying particular immediate thoughts and intentionally detaching from these thoughts.</t>
         </is>
       </c>
       <c r="D633" s="4" t="inlineStr">
         <is>
-          <t>physical behavioural opportunity</t>
+          <t>mental distancing</t>
         </is>
       </c>
       <c r="E633" s="4" t="n"/>
-      <c r="F633" s="4" t="inlineStr">
-        <is>
-          <t>Characteristics of a person's environment that involve the time available and influence the person's ability to enact a behaviour.</t>
-        </is>
-      </c>
-      <c r="G633" s="4" t="inlineStr">
-        <is>
-          <t>"Temporal" in the Needs-Opportunity-Abilities Model; "Time-space structures" in the Consumption as Social Practices; "Time (constraints)" in the Social Ecological Model of Behaviour Change</t>
-        </is>
-      </c>
+      <c r="F633" s="4" t="n"/>
+      <c r="G633" s="4" t="n"/>
       <c r="H633" s="4" t="n"/>
-      <c r="I633" s="4" t="n"/>
+      <c r="I633" s="4" t="inlineStr">
+        <is>
+          <t>targeted decentring</t>
+        </is>
+      </c>
       <c r="J633" s="4" t="n"/>
       <c r="K633" s="4" t="inlineStr">
         <is>
@@ -38029,29 +37997,29 @@
     <row r="634">
       <c r="A634" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050790</t>
+          <t>BCIO:050789</t>
         </is>
       </c>
       <c r="B634" s="4" t="inlineStr">
         <is>
-          <t>temporal orientation</t>
+          <t>technology availability</t>
         </is>
       </c>
       <c r="C634" s="4" t="inlineStr">
         <is>
-          <t>A &lt;mental disposition&gt; to appraise imagined future occurrences differently according to how far in the future they are judged to occur.</t>
+          <t>A &lt;behavioural opportunity&gt; that involves the extend to which technology is available in the environmental system.</t>
         </is>
       </c>
       <c r="D634" s="4" t="inlineStr">
         <is>
-          <t>mental disposition</t>
+          <t>behavioural opportunity</t>
         </is>
       </c>
       <c r="E634" s="4" t="n"/>
       <c r="F634" s="4" t="n"/>
       <c r="G634" s="4" t="inlineStr">
         <is>
-          <t>"Time orientation (near / far-sighted)" in the General Theory of Crime; "Time Preference" in the Rational Addiction Model</t>
+          <t>"Technology" in the Needs-Opportunity-Abilities Model</t>
         </is>
       </c>
       <c r="H634" s="4" t="n"/>
@@ -38091,29 +38059,33 @@
     <row r="635">
       <c r="A635" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050230</t>
+          <t>BCIO:006091</t>
         </is>
       </c>
       <c r="B635" s="4" t="inlineStr">
         <is>
-          <t>temporal orientation to the future</t>
+          <t>temporal behavioural opportunity</t>
         </is>
       </c>
       <c r="C635" s="4" t="inlineStr">
         <is>
-          <t>A &lt;temporal orientation&gt; to focus more on future than present outcomes.</t>
+          <t>A &lt;physical behavioural opportunity&gt; that involves the person having sufficient time or a suitable period.</t>
         </is>
       </c>
       <c r="D635" s="4" t="inlineStr">
         <is>
-          <t>temporal orientation</t>
+          <t>physical behavioural opportunity</t>
         </is>
       </c>
       <c r="E635" s="4" t="n"/>
-      <c r="F635" s="4" t="n"/>
+      <c r="F635" s="4" t="inlineStr">
+        <is>
+          <t>Characteristics of a person's environment that involve the time available and influence the person's ability to enact a behaviour.</t>
+        </is>
+      </c>
       <c r="G635" s="4" t="inlineStr">
         <is>
-          <t>"Future-oriented" in the Rational Addiction Model</t>
+          <t>"Temporal" in the Needs-Opportunity-Abilities Model; "Time-space structures" in the Consumption as Social Practices; "Time (constraints)" in the Social Ecological Model of Behaviour Change</t>
         </is>
       </c>
       <c r="H635" s="4" t="n"/>
@@ -38140,7 +38112,7 @@
       <c r="U635" s="4" t="n"/>
       <c r="V635" s="4" t="inlineStr">
         <is>
-          <t>PS; JD</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="W635" s="4" t="inlineStr">
@@ -38153,29 +38125,29 @@
     <row r="636">
       <c r="A636" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050231</t>
+          <t>BCIO:050790</t>
         </is>
       </c>
       <c r="B636" s="4" t="inlineStr">
         <is>
-          <t>temporal orientation to the present</t>
+          <t>temporal orientation</t>
         </is>
       </c>
       <c r="C636" s="4" t="inlineStr">
         <is>
-          <t>A &lt;temporal orientation&gt; to focus more on present than future outcomes.</t>
+          <t>A &lt;mental disposition&gt; to appraise imagined future occurrences differently according to how far in the future they are judged to occur.</t>
         </is>
       </c>
       <c r="D636" s="4" t="inlineStr">
         <is>
-          <t>temporal orientation</t>
+          <t>mental disposition</t>
         </is>
       </c>
       <c r="E636" s="4" t="n"/>
       <c r="F636" s="4" t="n"/>
       <c r="G636" s="4" t="inlineStr">
         <is>
-          <t>"Present-oriented" in the Rational Addiction Model; "Myopia" in the Rational Addiction Model</t>
+          <t>"Time orientation (near / far-sighted)" in the General Theory of Crime; "Time Preference" in the Rational Addiction Model</t>
         </is>
       </c>
       <c r="H636" s="4" t="n"/>
@@ -38213,73 +38185,93 @@
       <c r="X636" s="4" t="n"/>
     </row>
     <row r="637">
-      <c r="A637" t="inlineStr">
-        <is>
-          <t>MF:0000013</t>
-        </is>
-      </c>
-      <c r="B637" t="inlineStr">
-        <is>
-          <t>thinking</t>
-        </is>
-      </c>
-      <c r="C637" t="inlineStr">
-        <is>
-          <t>A &lt;cognitive process&gt; that involves the manipulation of mental language and/or mental images.</t>
-        </is>
-      </c>
-      <c r="D637" t="inlineStr">
-        <is>
-          <t>cognitive process</t>
-        </is>
-      </c>
-      <c r="K637" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S637" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V637" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W637" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="A637" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050230</t>
+        </is>
+      </c>
+      <c r="B637" s="4" t="inlineStr">
+        <is>
+          <t>temporal orientation to the future</t>
+        </is>
+      </c>
+      <c r="C637" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;temporal orientation&gt; to focus more on future than present outcomes.</t>
+        </is>
+      </c>
+      <c r="D637" s="4" t="inlineStr">
+        <is>
+          <t>temporal orientation</t>
+        </is>
+      </c>
+      <c r="E637" s="4" t="n"/>
+      <c r="F637" s="4" t="n"/>
+      <c r="G637" s="4" t="inlineStr">
+        <is>
+          <t>"Future-oriented" in the Rational Addiction Model</t>
+        </is>
+      </c>
+      <c r="H637" s="4" t="n"/>
+      <c r="I637" s="4" t="n"/>
+      <c r="J637" s="4" t="n"/>
+      <c r="K637" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L637" s="4" t="n"/>
+      <c r="M637" s="4" t="n"/>
+      <c r="N637" s="4" t="n"/>
+      <c r="O637" s="4" t="n"/>
+      <c r="P637" s="4" t="n"/>
+      <c r="Q637" s="4" t="n"/>
+      <c r="R637" s="4" t="n"/>
+      <c r="S637" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T637" s="4" t="n"/>
+      <c r="U637" s="4" t="n"/>
+      <c r="V637" s="4" t="inlineStr">
+        <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W637" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X637" s="4" t="n"/>
     </row>
     <row r="638">
       <c r="A638" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050791</t>
+          <t>BCIO:050231</t>
         </is>
       </c>
       <c r="B638" s="4" t="inlineStr">
         <is>
-          <t>threat appraisal</t>
+          <t>temporal orientation to the present</t>
         </is>
       </c>
       <c r="C638" s="4" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is about belief about threat expressed as the likelihood of a potentially harmful occurrence weighted by the severity of the harm.</t>
+          <t>A &lt;temporal orientation&gt; to focus more on present than future outcomes.</t>
         </is>
       </c>
       <c r="D638" s="4" t="inlineStr">
         <is>
-          <t>data item</t>
+          <t>temporal orientation</t>
         </is>
       </c>
       <c r="E638" s="4" t="n"/>
       <c r="F638" s="4" t="n"/>
       <c r="G638" s="4" t="inlineStr">
         <is>
-          <t>"Threat appraisal" in the Protection Motivation Theory</t>
+          <t>"Present-oriented" in the Rational Addiction Model; "Myopia" in the Rational Addiction Model</t>
         </is>
       </c>
       <c r="H638" s="4" t="n"/>
@@ -38317,93 +38309,73 @@
       <c r="X638" s="4" t="n"/>
     </row>
     <row r="639">
-      <c r="A639" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050884</t>
-        </is>
-      </c>
-      <c r="B639" s="4" t="inlineStr">
-        <is>
-          <t>total internal influence on behaviour</t>
-        </is>
-      </c>
-      <c r="C639" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;bodily disposition&gt; that is the aggregate of internal influences on behaviour.</t>
-        </is>
-      </c>
-      <c r="D639" s="4" t="inlineStr">
-        <is>
-          <t>bodily disposition</t>
-        </is>
-      </c>
-      <c r="E639" s="4" t="n"/>
-      <c r="F639" s="4" t="n"/>
-      <c r="G639" s="4" t="inlineStr">
-        <is>
-          <t>"Internal factors" in the Model of Pro-Environmental Behavior</t>
-        </is>
-      </c>
-      <c r="H639" s="4" t="n"/>
-      <c r="I639" s="4" t="n"/>
-      <c r="J639" s="4" t="n"/>
-      <c r="K639" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L639" s="4" t="n"/>
-      <c r="M639" s="4" t="n"/>
-      <c r="N639" s="4" t="n"/>
-      <c r="O639" s="4" t="n"/>
-      <c r="P639" s="4" t="n"/>
-      <c r="Q639" s="4" t="n"/>
-      <c r="R639" s="4" t="n"/>
-      <c r="S639" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T639" s="4" t="n"/>
-      <c r="U639" s="4" t="n"/>
-      <c r="V639" s="4" t="inlineStr">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>MF:0000013</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>thinking</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>A &lt;cognitive process&gt; that involves the manipulation of mental language and/or mental images.</t>
+        </is>
+      </c>
+      <c r="D639" t="inlineStr">
+        <is>
+          <t>cognitive process</t>
+        </is>
+      </c>
+      <c r="K639" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S639" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V639" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W639" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X639" s="4" t="n"/>
+      <c r="W639" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="640">
       <c r="A640" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050792</t>
+          <t>BCIO:050791</t>
         </is>
       </c>
       <c r="B640" s="4" t="inlineStr">
         <is>
-          <t>traditional personal value</t>
+          <t>threat appraisal</t>
         </is>
       </c>
       <c r="C640" s="4" t="inlineStr">
         <is>
-          <t>A &lt;personal value&gt; that involves regarding long-standing social customs as fundamentally important in life.</t>
+          <t>A &lt;data item&gt; that is about belief about threat expressed as the likelihood of a potentially harmful occurrence weighted by the severity of the harm.</t>
         </is>
       </c>
       <c r="D640" s="4" t="inlineStr">
         <is>
-          <t>personal value</t>
+          <t>data item</t>
         </is>
       </c>
       <c r="E640" s="4" t="n"/>
       <c r="F640" s="4" t="n"/>
       <c r="G640" s="4" t="inlineStr">
         <is>
-          <t>"Traditional values" in the Value Belief Norm Theory; "Belief (prosocial / antisocial)" in the Social Development Model</t>
+          <t>"Threat appraisal" in the Protection Motivation Theory</t>
         </is>
       </c>
       <c r="H640" s="4" t="n"/>
@@ -38443,38 +38415,34 @@
     <row r="641">
       <c r="A641" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050885</t>
+          <t>BCIO:050884</t>
         </is>
       </c>
       <c r="B641" s="4" t="inlineStr">
         <is>
-          <t>underestimated perceived descriptive norm</t>
+          <t>total internal influence on behaviour</t>
         </is>
       </c>
       <c r="C641" s="4" t="inlineStr">
         <is>
-          <t>A &lt;perceived descriptive behavioural norm&gt; in which the prevalence of a behaviour is underestimated.</t>
+          <t>A &lt;bodily disposition&gt; that is the aggregate of internal influences on behaviour.</t>
         </is>
       </c>
       <c r="D641" s="4" t="inlineStr">
         <is>
-          <t>perceived descriptive behavioural norm</t>
+          <t>bodily disposition</t>
         </is>
       </c>
       <c r="E641" s="4" t="n"/>
       <c r="F641" s="4" t="n"/>
       <c r="G641" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"False uniqueness" in the Social Norms Theory </t>
+          <t>"Internal factors" in the Model of Pro-Environmental Behavior</t>
         </is>
       </c>
       <c r="H641" s="4" t="n"/>
       <c r="I641" s="4" t="n"/>
-      <c r="J641" s="4" t="inlineStr">
-        <is>
-          <t>This is the belief of an individual.</t>
-        </is>
-      </c>
+      <c r="J641" s="4" t="n"/>
       <c r="K641" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -38496,105 +38464,113 @@
       <c r="U641" s="4" t="n"/>
       <c r="V641" s="4" t="inlineStr">
         <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W641" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X641" s="4" t="n"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050792</t>
+        </is>
+      </c>
+      <c r="B642" s="4" t="inlineStr">
+        <is>
+          <t>traditional personal value</t>
+        </is>
+      </c>
+      <c r="C642" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;personal value&gt; that involves regarding long-standing social customs as fundamentally important in life.</t>
+        </is>
+      </c>
+      <c r="D642" s="4" t="inlineStr">
+        <is>
+          <t>personal value</t>
+        </is>
+      </c>
+      <c r="E642" s="4" t="n"/>
+      <c r="F642" s="4" t="n"/>
+      <c r="G642" s="4" t="inlineStr">
+        <is>
+          <t>"Traditional values" in the Value Belief Norm Theory; "Belief (prosocial / antisocial)" in the Social Development Model</t>
+        </is>
+      </c>
+      <c r="H642" s="4" t="n"/>
+      <c r="I642" s="4" t="n"/>
+      <c r="J642" s="4" t="n"/>
+      <c r="K642" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L642" s="4" t="n"/>
+      <c r="M642" s="4" t="n"/>
+      <c r="N642" s="4" t="n"/>
+      <c r="O642" s="4" t="n"/>
+      <c r="P642" s="4" t="n"/>
+      <c r="Q642" s="4" t="n"/>
+      <c r="R642" s="4" t="n"/>
+      <c r="S642" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T642" s="4" t="n"/>
+      <c r="U642" s="4" t="n"/>
+      <c r="V642" s="4" t="inlineStr">
+        <is>
           <t>PS; JD</t>
         </is>
       </c>
-      <c r="W641" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X641" s="4" t="n"/>
-    </row>
-    <row r="642">
-      <c r="A642" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050267</t>
-        </is>
-      </c>
-      <c r="B642" s="3" t="inlineStr">
-        <is>
-          <t>uniform process aggregate</t>
-        </is>
-      </c>
-      <c r="C642" s="3" t="inlineStr">
-        <is>
-          <t>A process aggregate whose member parts are of the same type.</t>
-        </is>
-      </c>
-      <c r="D642" s="3" t="inlineStr">
-        <is>
-          <t>process aggregate</t>
-        </is>
-      </c>
-      <c r="E642" s="3" t="n"/>
-      <c r="F642" s="3" t="n"/>
-      <c r="G642" s="3" t="n"/>
-      <c r="H642" s="3" t="n"/>
-      <c r="I642" s="3" t="n"/>
-      <c r="J642" s="3" t="n"/>
-      <c r="K642" s="3" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L642" s="3" t="n"/>
-      <c r="M642" s="3" t="n"/>
-      <c r="N642" s="3" t="n"/>
-      <c r="O642" s="3" t="n"/>
-      <c r="P642" s="3" t="n"/>
-      <c r="Q642" s="3" t="n"/>
-      <c r="R642" s="3" t="n"/>
-      <c r="S642" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="T642" s="3" t="n"/>
-      <c r="U642" s="3" t="n"/>
-      <c r="V642" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W642" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X642" s="3" t="n"/>
+      <c r="W642" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X642" s="4" t="n"/>
     </row>
     <row r="643">
       <c r="A643" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050793</t>
+          <t>BCIO:050885</t>
         </is>
       </c>
       <c r="B643" s="4" t="inlineStr">
         <is>
-          <t>utility maximisation disposition</t>
+          <t>underestimated perceived descriptive norm</t>
         </is>
       </c>
       <c r="C643" s="4" t="inlineStr">
         <is>
-          <t>A &lt;mental disposition&gt; to behave in a way that seeks to maximise the net positive consequences of behaviour.</t>
+          <t>A &lt;perceived descriptive behavioural norm&gt; in which the prevalence of a behaviour is underestimated.</t>
         </is>
       </c>
       <c r="D643" s="4" t="inlineStr">
         <is>
-          <t>mental disposition</t>
+          <t>perceived descriptive behavioural norm</t>
         </is>
       </c>
       <c r="E643" s="4" t="n"/>
       <c r="F643" s="4" t="n"/>
       <c r="G643" s="4" t="inlineStr">
         <is>
-          <t>"Rationality" in the Rational Addiction Model</t>
+          <t xml:space="preserve">"False uniqueness" in the Social Norms Theory </t>
         </is>
       </c>
       <c r="H643" s="4" t="n"/>
       <c r="I643" s="4" t="n"/>
-      <c r="J643" s="4" t="n"/>
+      <c r="J643" s="4" t="inlineStr">
+        <is>
+          <t>This is the belief of an individual.</t>
+        </is>
+      </c>
       <c r="K643" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -38627,91 +38603,91 @@
       <c r="X643" s="4" t="n"/>
     </row>
     <row r="644">
-      <c r="A644" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:006107</t>
-        </is>
-      </c>
-      <c r="B644" s="4" t="inlineStr">
-        <is>
-          <t>value-congruent self-regulation</t>
-        </is>
-      </c>
-      <c r="C644" s="4" t="inlineStr">
-        <is>
-          <t>&lt;Self-regulation of behaviour&gt; undertaken to achieve consistency between one's values and the behaviour performed.</t>
-        </is>
-      </c>
-      <c r="D644" s="4" t="inlineStr">
-        <is>
-          <t>self-regulation of behaviour</t>
-        </is>
-      </c>
-      <c r="E644" s="4" t="n"/>
-      <c r="F644" s="4" t="n"/>
-      <c r="G644" s="4" t="inlineStr">
-        <is>
-          <t>"Integrated internalisation and Self-Regulation of Health Behaviour" in the Health Behaviour Internalisation Model</t>
-        </is>
-      </c>
-      <c r="H644" s="4" t="n"/>
-      <c r="I644" s="4" t="n"/>
-      <c r="J644" s="4" t="n"/>
-      <c r="K644" s="4" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L644" s="4" t="n"/>
-      <c r="M644" s="4" t="n"/>
-      <c r="N644" s="4" t="n"/>
-      <c r="O644" s="4" t="n"/>
-      <c r="P644" s="4" t="n"/>
-      <c r="Q644" s="4" t="n"/>
-      <c r="R644" s="4" t="n"/>
-      <c r="S644" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T644" s="4" t="n"/>
-      <c r="U644" s="4" t="n"/>
-      <c r="V644" s="4" t="inlineStr">
+      <c r="A644" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050267</t>
+        </is>
+      </c>
+      <c r="B644" s="3" t="inlineStr">
+        <is>
+          <t>uniform process aggregate</t>
+        </is>
+      </c>
+      <c r="C644" s="3" t="inlineStr">
+        <is>
+          <t>A process aggregate whose member parts are of the same type.</t>
+        </is>
+      </c>
+      <c r="D644" s="3" t="inlineStr">
+        <is>
+          <t>process aggregate</t>
+        </is>
+      </c>
+      <c r="E644" s="3" t="n"/>
+      <c r="F644" s="3" t="n"/>
+      <c r="G644" s="3" t="n"/>
+      <c r="H644" s="3" t="n"/>
+      <c r="I644" s="3" t="n"/>
+      <c r="J644" s="3" t="n"/>
+      <c r="K644" s="3" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L644" s="3" t="n"/>
+      <c r="M644" s="3" t="n"/>
+      <c r="N644" s="3" t="n"/>
+      <c r="O644" s="3" t="n"/>
+      <c r="P644" s="3" t="n"/>
+      <c r="Q644" s="3" t="n"/>
+      <c r="R644" s="3" t="n"/>
+      <c r="S644" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="T644" s="3" t="n"/>
+      <c r="U644" s="3" t="n"/>
+      <c r="V644" s="3" t="inlineStr">
         <is>
           <t>PS</t>
         </is>
       </c>
-      <c r="W644" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X644" s="4" t="n"/>
+      <c r="W644" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X644" s="3" t="n"/>
     </row>
     <row r="645">
       <c r="A645" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050794</t>
+          <t>BCIO:050793</t>
         </is>
       </c>
       <c r="B645" s="4" t="inlineStr">
         <is>
-          <t>vicarious learning</t>
+          <t>utility maximisation disposition</t>
         </is>
       </c>
       <c r="C645" s="4" t="inlineStr">
         <is>
-          <t>&lt;Observational learning&gt; that occurs through observing the consequences of the actions of others.</t>
+          <t>A &lt;mental disposition&gt; to behave in a way that seeks to maximise the net positive consequences of behaviour.</t>
         </is>
       </c>
       <c r="D645" s="4" t="inlineStr">
         <is>
-          <t>observational learning</t>
+          <t>mental disposition</t>
         </is>
       </c>
       <c r="E645" s="4" t="n"/>
       <c r="F645" s="4" t="n"/>
-      <c r="G645" s="4" t="n"/>
+      <c r="G645" s="4" t="inlineStr">
+        <is>
+          <t>"Rationality" in the Rational Addiction Model</t>
+        </is>
+      </c>
       <c r="H645" s="4" t="n"/>
       <c r="I645" s="4" t="n"/>
       <c r="J645" s="4" t="n"/>
@@ -38736,7 +38712,7 @@
       <c r="U645" s="4" t="n"/>
       <c r="V645" s="4" t="inlineStr">
         <is>
-          <t>PS</t>
+          <t>PS; JD</t>
         </is>
       </c>
       <c r="W645" s="4" t="inlineStr">
@@ -38749,29 +38725,29 @@
     <row r="646">
       <c r="A646" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050795</t>
+          <t>BCIO:006107</t>
         </is>
       </c>
       <c r="B646" s="4" t="inlineStr">
         <is>
-          <t>vicarious learning capability</t>
+          <t>value-congruent self-regulation</t>
         </is>
       </c>
       <c r="C646" s="4" t="inlineStr">
         <is>
-          <t>An &lt;observational learning capability&gt; through the observing the consequences of the actions of others.</t>
+          <t>&lt;Self-regulation of behaviour&gt; undertaken to achieve consistency between one's values and the behaviour performed.</t>
         </is>
       </c>
       <c r="D646" s="4" t="inlineStr">
         <is>
-          <t>observational learning capability</t>
+          <t>self-regulation of behaviour</t>
         </is>
       </c>
       <c r="E646" s="4" t="n"/>
       <c r="F646" s="4" t="n"/>
       <c r="G646" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">"Vicarious learning capability" in the Social Cognitive Theory </t>
+          <t>"Integrated internalisation and Self-Regulation of Health Behaviour" in the Health Behaviour Internalisation Model</t>
         </is>
       </c>
       <c r="H646" s="4" t="n"/>
@@ -38798,7 +38774,7 @@
       <c r="U646" s="4" t="n"/>
       <c r="V646" s="4" t="inlineStr">
         <is>
-          <t>PS; JD</t>
+          <t>PS</t>
         </is>
       </c>
       <c r="W646" s="4" t="inlineStr">
@@ -38809,78 +38785,89 @@
       <c r="X646" s="4" t="n"/>
     </row>
     <row r="647">
-      <c r="A647" t="inlineStr">
-        <is>
-          <t>MF:0000045</t>
-        </is>
-      </c>
-      <c r="B647" t="inlineStr">
-        <is>
-          <t>wanting</t>
-        </is>
-      </c>
-      <c r="C647" t="inlineStr">
-        <is>
-          <t>A &lt;mental process&gt; that involves thinking about a state of affairs that is not yet the case together with a desire for that state of affairs to come about.</t>
-        </is>
-      </c>
-      <c r="D647" t="inlineStr">
-        <is>
-          <t>mental process</t>
-        </is>
-      </c>
-      <c r="G647" t="inlineStr">
-        <is>
-          <t>"Temptation" in the Transtheoretical Model; "Hedonic values" in the Goal-Framing Theory; "Desire" in the Action Theory Model of Consumption; "Desires" in the Social Influence Model; "Decision-making and participation" in the  Social Influence Model</t>
-        </is>
-      </c>
-      <c r="K647" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="S647" t="inlineStr">
-        <is>
-          <t>External</t>
-        </is>
-      </c>
-      <c r="V647" t="inlineStr">
-        <is>
-          <t>PS; JD</t>
-        </is>
-      </c>
-      <c r="W647" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+      <c r="A647" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050794</t>
+        </is>
+      </c>
+      <c r="B647" s="4" t="inlineStr">
+        <is>
+          <t>vicarious learning</t>
+        </is>
+      </c>
+      <c r="C647" s="4" t="inlineStr">
+        <is>
+          <t>&lt;Observational learning&gt; that occurs through observing the consequences of the actions of others.</t>
+        </is>
+      </c>
+      <c r="D647" s="4" t="inlineStr">
+        <is>
+          <t>observational learning</t>
+        </is>
+      </c>
+      <c r="E647" s="4" t="n"/>
+      <c r="F647" s="4" t="n"/>
+      <c r="G647" s="4" t="n"/>
+      <c r="H647" s="4" t="n"/>
+      <c r="I647" s="4" t="n"/>
+      <c r="J647" s="4" t="n"/>
+      <c r="K647" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L647" s="4" t="n"/>
+      <c r="M647" s="4" t="n"/>
+      <c r="N647" s="4" t="n"/>
+      <c r="O647" s="4" t="n"/>
+      <c r="P647" s="4" t="n"/>
+      <c r="Q647" s="4" t="n"/>
+      <c r="R647" s="4" t="n"/>
+      <c r="S647" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T647" s="4" t="n"/>
+      <c r="U647" s="4" t="n"/>
+      <c r="V647" s="4" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W647" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X647" s="4" t="n"/>
     </row>
     <row r="648">
       <c r="A648" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050796</t>
+          <t>BCIO:050795</t>
         </is>
       </c>
       <c r="B648" s="4" t="inlineStr">
         <is>
-          <t>well-specified goal</t>
+          <t>vicarious learning capability</t>
         </is>
       </c>
       <c r="C648" s="4" t="inlineStr">
         <is>
-          <t>A &lt;goal&gt; that is specified in sufficient detail for it to be clear when the goal has been achieved.</t>
+          <t>An &lt;observational learning capability&gt; through the observing the consequences of the actions of others.</t>
         </is>
       </c>
       <c r="D648" s="4" t="inlineStr">
         <is>
-          <t>goal</t>
+          <t>observational learning capability</t>
         </is>
       </c>
       <c r="E648" s="4" t="n"/>
       <c r="F648" s="4" t="n"/>
       <c r="G648" s="4" t="inlineStr">
         <is>
-          <t>"Goal specificity" in the Goal Setting Theory</t>
+          <t xml:space="preserve">"Vicarious learning capability" in the Social Cognitive Theory </t>
         </is>
       </c>
       <c r="H648" s="4" t="n"/>
@@ -38918,98 +38905,83 @@
       <c r="X648" s="4" t="n"/>
     </row>
     <row r="649">
-      <c r="A649" s="3" t="inlineStr">
-        <is>
-          <t>BCIO:050797</t>
-        </is>
-      </c>
-      <c r="B649" s="3" t="inlineStr">
-        <is>
-          <t>wider community behavioural consequence</t>
-        </is>
-      </c>
-      <c r="C649" s="3" t="inlineStr">
-        <is>
-          <t>A &lt;social behavioural consequence&gt; that is beyond the person’s family.</t>
-        </is>
-      </c>
-      <c r="D649" s="3" t="inlineStr">
-        <is>
-          <t>social behavioural consequence</t>
-        </is>
-      </c>
-      <c r="E649" s="3" t="n"/>
-      <c r="F649" s="3" t="n"/>
-      <c r="G649" s="3" t="n"/>
-      <c r="H649" s="3" t="n"/>
-      <c r="I649" s="3" t="n"/>
-      <c r="J649" s="3" t="n"/>
-      <c r="K649" s="3" t="inlineStr">
-        <is>
-          <t>Mechanisms of action</t>
-        </is>
-      </c>
-      <c r="L649" s="3" t="n"/>
-      <c r="M649" s="3" t="n"/>
-      <c r="N649" s="3" t="n"/>
-      <c r="O649" s="3" t="n"/>
-      <c r="P649" s="3" t="n"/>
-      <c r="Q649" s="3" t="n"/>
-      <c r="R649" s="3" t="n"/>
-      <c r="S649" s="3" t="inlineStr">
-        <is>
-          <t>Obsolete</t>
-        </is>
-      </c>
-      <c r="T649" s="3" t="n"/>
-      <c r="U649" s="3" t="n"/>
-      <c r="V649" s="3" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
-      <c r="W649" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="X649" s="3" t="n"/>
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>MF:0000045</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>wanting</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>A &lt;mental process&gt; that involves thinking about a state of affairs that is not yet the case together with a desire for that state of affairs to come about.</t>
+        </is>
+      </c>
+      <c r="D649" t="inlineStr">
+        <is>
+          <t>mental process</t>
+        </is>
+      </c>
+      <c r="G649" t="inlineStr">
+        <is>
+          <t>"Temptation" in the Transtheoretical Model; "Hedonic values" in the Goal-Framing Theory; "Desire" in the Action Theory Model of Consumption; "Desires" in the Social Influence Model; "Decision-making and participation" in the  Social Influence Model</t>
+        </is>
+      </c>
+      <c r="K649" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="S649" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="V649" t="inlineStr">
+        <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W649" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="650">
       <c r="A650" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050798</t>
+          <t>BCIO:050796</t>
         </is>
       </c>
       <c r="B650" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">willingness to adopt new behaviours </t>
+          <t>well-specified goal</t>
         </is>
       </c>
       <c r="C650" s="4" t="inlineStr">
         <is>
-          <t>A &lt;willingness to change behaviour&gt; to adopt new behaviours.</t>
+          <t>A &lt;goal&gt; that is specified in sufficient detail for it to be clear when the goal has been achieved.</t>
         </is>
       </c>
       <c r="D650" s="4" t="inlineStr">
         <is>
-          <t>willingness to change behaviour</t>
+          <t>goal</t>
         </is>
       </c>
       <c r="E650" s="4" t="n"/>
       <c r="F650" s="4" t="n"/>
       <c r="G650" s="4" t="inlineStr">
         <is>
-          <t>"Innovators" in the Diffusion of Innovations; "Early majority" in the Diffusion of Innovations; "Early adopters" in the Diffusion of Innovations; "Late majority" in the Diffusion of Innovations; "Laggards" in the Diffusion of Innovations</t>
+          <t>"Goal specificity" in the Goal Setting Theory</t>
         </is>
       </c>
       <c r="H650" s="4" t="n"/>
       <c r="I650" s="4" t="n"/>
-      <c r="J650" s="4" t="inlineStr">
-        <is>
-          <t>This is a dimension that can be subdivided into very high, high, medium, low and very low.</t>
-        </is>
-      </c>
+      <c r="J650" s="4" t="n"/>
       <c r="K650" s="4" t="inlineStr">
         <is>
           <t>Mechanisms of action</t>
@@ -39042,85 +39014,103 @@
       <c r="X650" s="4" t="n"/>
     </row>
     <row r="651">
-      <c r="A651" s="4" t="inlineStr">
-        <is>
-          <t>BCIO:050951</t>
-        </is>
-      </c>
-      <c r="B651" s="4" t="inlineStr">
-        <is>
-          <t>willingness to cease behaviour</t>
-        </is>
-      </c>
-      <c r="C651" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;willingness to change behaviour&gt; regarding the cessation of behaviours.</t>
-        </is>
-      </c>
-      <c r="D651" s="4" t="inlineStr">
-        <is>
-          <t>willingness to change behaviour</t>
-        </is>
-      </c>
-      <c r="E651" s="4" t="n"/>
-      <c r="F651" s="4" t="n"/>
-      <c r="G651" s="4" t="n"/>
-      <c r="H651" s="4" t="n"/>
-      <c r="I651" s="4" t="n"/>
-      <c r="J651" s="4" t="n"/>
-      <c r="K651" s="4" t="n"/>
-      <c r="L651" s="4" t="n"/>
-      <c r="M651" s="4" t="n"/>
-      <c r="N651" s="4" t="n"/>
-      <c r="O651" s="4" t="n"/>
-      <c r="P651" s="4" t="n"/>
-      <c r="Q651" s="4" t="n"/>
-      <c r="R651" s="4" t="n"/>
-      <c r="S651" s="4" t="inlineStr">
-        <is>
-          <t>Published</t>
-        </is>
-      </c>
-      <c r="T651" s="4" t="n"/>
-      <c r="U651" s="4" t="n"/>
-      <c r="V651" s="4" t="inlineStr">
-        <is>
-          <t>MB</t>
-        </is>
-      </c>
-      <c r="W651" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X651" s="4" t="n"/>
+      <c r="A651" s="3" t="inlineStr">
+        <is>
+          <t>BCIO:050797</t>
+        </is>
+      </c>
+      <c r="B651" s="3" t="inlineStr">
+        <is>
+          <t>wider community behavioural consequence</t>
+        </is>
+      </c>
+      <c r="C651" s="3" t="inlineStr">
+        <is>
+          <t>A &lt;social behavioural consequence&gt; that is beyond the person’s family.</t>
+        </is>
+      </c>
+      <c r="D651" s="3" t="inlineStr">
+        <is>
+          <t>social behavioural consequence</t>
+        </is>
+      </c>
+      <c r="E651" s="3" t="n"/>
+      <c r="F651" s="3" t="n"/>
+      <c r="G651" s="3" t="n"/>
+      <c r="H651" s="3" t="n"/>
+      <c r="I651" s="3" t="n"/>
+      <c r="J651" s="3" t="n"/>
+      <c r="K651" s="3" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
+      <c r="L651" s="3" t="n"/>
+      <c r="M651" s="3" t="n"/>
+      <c r="N651" s="3" t="n"/>
+      <c r="O651" s="3" t="n"/>
+      <c r="P651" s="3" t="n"/>
+      <c r="Q651" s="3" t="n"/>
+      <c r="R651" s="3" t="n"/>
+      <c r="S651" s="3" t="inlineStr">
+        <is>
+          <t>Obsolete</t>
+        </is>
+      </c>
+      <c r="T651" s="3" t="n"/>
+      <c r="U651" s="3" t="n"/>
+      <c r="V651" s="3" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="W651" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X651" s="3" t="n"/>
     </row>
     <row r="652">
       <c r="A652" s="4" t="inlineStr">
         <is>
-          <t>BCIO:050952</t>
+          <t>BCIO:050798</t>
         </is>
       </c>
       <c r="B652" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">willingness to adopt new behaviours </t>
+        </is>
+      </c>
+      <c r="C652" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;willingness to change behaviour&gt; to adopt new behaviours.</t>
+        </is>
+      </c>
+      <c r="D652" s="4" t="inlineStr">
+        <is>
           <t>willingness to change behaviour</t>
-        </is>
-      </c>
-      <c r="C652" s="4" t="inlineStr">
-        <is>
-          <t>A &lt;bodily disposition&gt; to change one's behaviour.</t>
-        </is>
-      </c>
-      <c r="D652" s="4" t="inlineStr">
-        <is>
-          <t>bodily disposition</t>
         </is>
       </c>
       <c r="E652" s="4" t="n"/>
       <c r="F652" s="4" t="n"/>
-      <c r="G652" s="4" t="n"/>
+      <c r="G652" s="4" t="inlineStr">
+        <is>
+          <t>"Innovators" in the Diffusion of Innovations; "Early majority" in the Diffusion of Innovations; "Early adopters" in the Diffusion of Innovations; "Late majority" in the Diffusion of Innovations; "Laggards" in the Diffusion of Innovations</t>
+        </is>
+      </c>
       <c r="H652" s="4" t="n"/>
       <c r="I652" s="4" t="n"/>
-      <c r="J652" s="4" t="n"/>
-      <c r="K652" s="4" t="n"/>
+      <c r="J652" s="4" t="inlineStr">
+        <is>
+          <t>This is a dimension that can be subdivided into very high, high, medium, low and very low.</t>
+        </is>
+      </c>
+      <c r="K652" s="4" t="inlineStr">
+        <is>
+          <t>Mechanisms of action</t>
+        </is>
+      </c>
       <c r="L652" s="4" t="n"/>
       <c r="M652" s="4" t="n"/>
       <c r="N652" s="4" t="n"/>
@@ -39137,13 +39127,119 @@
       <c r="U652" s="4" t="n"/>
       <c r="V652" s="4" t="inlineStr">
         <is>
+          <t>PS; JD</t>
+        </is>
+      </c>
+      <c r="W652" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="X652" s="4" t="n"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050951</t>
+        </is>
+      </c>
+      <c r="B653" s="4" t="inlineStr">
+        <is>
+          <t>willingness to cease behaviour</t>
+        </is>
+      </c>
+      <c r="C653" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;willingness to change behaviour&gt; regarding the cessation of behaviours.</t>
+        </is>
+      </c>
+      <c r="D653" s="4" t="inlineStr">
+        <is>
+          <t>willingness to change behaviour</t>
+        </is>
+      </c>
+      <c r="E653" s="4" t="n"/>
+      <c r="F653" s="4" t="n"/>
+      <c r="G653" s="4" t="n"/>
+      <c r="H653" s="4" t="n"/>
+      <c r="I653" s="4" t="n"/>
+      <c r="J653" s="4" t="n"/>
+      <c r="K653" s="4" t="n"/>
+      <c r="L653" s="4" t="n"/>
+      <c r="M653" s="4" t="n"/>
+      <c r="N653" s="4" t="n"/>
+      <c r="O653" s="4" t="n"/>
+      <c r="P653" s="4" t="n"/>
+      <c r="Q653" s="4" t="n"/>
+      <c r="R653" s="4" t="n"/>
+      <c r="S653" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T653" s="4" t="n"/>
+      <c r="U653" s="4" t="n"/>
+      <c r="V653" s="4" t="inlineStr">
+        <is>
           <t>MB</t>
         </is>
       </c>
-      <c r="W652" s="4" t="n">
+      <c r="W653" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="X652" s="4" t="n"/>
+      <c r="X653" s="4" t="n"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="4" t="inlineStr">
+        <is>
+          <t>BCIO:050952</t>
+        </is>
+      </c>
+      <c r="B654" s="4" t="inlineStr">
+        <is>
+          <t>willingness to change behaviour</t>
+        </is>
+      </c>
+      <c r="C654" s="4" t="inlineStr">
+        <is>
+          <t>A &lt;bodily disposition&gt; to change one's behaviour.</t>
+        </is>
+      </c>
+      <c r="D654" s="4" t="inlineStr">
+        <is>
+          <t>bodily disposition</t>
+        </is>
+      </c>
+      <c r="E654" s="4" t="n"/>
+      <c r="F654" s="4" t="n"/>
+      <c r="G654" s="4" t="n"/>
+      <c r="H654" s="4" t="n"/>
+      <c r="I654" s="4" t="n"/>
+      <c r="J654" s="4" t="n"/>
+      <c r="K654" s="4" t="n"/>
+      <c r="L654" s="4" t="n"/>
+      <c r="M654" s="4" t="n"/>
+      <c r="N654" s="4" t="n"/>
+      <c r="O654" s="4" t="n"/>
+      <c r="P654" s="4" t="n"/>
+      <c r="Q654" s="4" t="n"/>
+      <c r="R654" s="4" t="n"/>
+      <c r="S654" s="4" t="inlineStr">
+        <is>
+          <t>Published</t>
+        </is>
+      </c>
+      <c r="T654" s="4" t="n"/>
+      <c r="U654" s="4" t="n"/>
+      <c r="V654" s="4" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="W654" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X654" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>